<commit_message>
generated all partB results
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vanessa\Documents\Uni\Bachelor-Thesis\BachelorThesis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{18DCDD51-FA93-49D2-BAF8-D11126C39712}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30350997-3BBF-49AB-916C-212AA2CBCFFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{2A4234DB-3A22-4351-83C3-53CA1AE1142A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="677" uniqueCount="102">
   <si>
     <t>Benchmarking results LLMs</t>
   </si>
@@ -339,6 +339,9 @@
   </si>
   <si>
     <t>parsing + area feasibility check</t>
+  </si>
+  <si>
+    <t>Part B</t>
   </si>
 </sst>
 </file>
@@ -759,7 +762,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9626A942-19B5-4B39-BBE2-849051787A6F}">
-  <dimension ref="A1:O84"/>
+  <dimension ref="A1:O184"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="15.28515625" customWidth="1"/>
@@ -3543,6 +3546,1632 @@
         <v>78</v>
       </c>
     </row>
+    <row r="96" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="97" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A97">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="99" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A99" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C99" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D99" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E99" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G99" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H99" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I99" s="1"/>
+      <c r="J99" s="1"/>
+      <c r="K99" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="L99" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="M99" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="N99" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O99" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="100" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A100" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B100" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D100" s="2">
+        <v>1</v>
+      </c>
+      <c r="E100" s="3"/>
+      <c r="F100" s="3"/>
+      <c r="G100" s="2"/>
+      <c r="H100" s="2"/>
+      <c r="I100" s="2"/>
+      <c r="J100" s="2"/>
+      <c r="K100" s="3"/>
+      <c r="L100" s="3"/>
+      <c r="M100" s="3"/>
+      <c r="N100" s="3"/>
+      <c r="O100" s="3"/>
+    </row>
+    <row r="101" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A101" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C101" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D101" s="4">
+        <v>1</v>
+      </c>
+      <c r="E101" s="5"/>
+      <c r="F101" s="6"/>
+      <c r="G101" s="4"/>
+      <c r="H101" s="4"/>
+      <c r="I101" s="4"/>
+      <c r="J101" s="4"/>
+      <c r="K101" s="5"/>
+      <c r="L101" s="5"/>
+      <c r="M101" s="4"/>
+      <c r="N101" s="4"/>
+      <c r="O101" s="4"/>
+    </row>
+    <row r="102" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A102" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D102" s="2">
+        <v>1</v>
+      </c>
+      <c r="E102" s="3"/>
+      <c r="F102" s="3"/>
+      <c r="G102" s="2"/>
+      <c r="H102" s="2"/>
+      <c r="I102" s="2"/>
+      <c r="J102" s="2"/>
+      <c r="K102" s="3"/>
+      <c r="L102" s="3"/>
+      <c r="M102" s="3"/>
+      <c r="N102" s="3"/>
+      <c r="O102" s="3"/>
+    </row>
+    <row r="103" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A103" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C103" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103" s="4">
+        <v>1</v>
+      </c>
+      <c r="E103" s="5"/>
+      <c r="F103" s="4"/>
+      <c r="G103" s="4"/>
+      <c r="H103" s="4"/>
+      <c r="I103" s="4"/>
+      <c r="J103" s="4"/>
+      <c r="K103" s="5"/>
+      <c r="L103" s="5"/>
+      <c r="M103" s="4"/>
+      <c r="N103" s="4"/>
+      <c r="O103" s="4"/>
+    </row>
+    <row r="104" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A104" s="1"/>
+      <c r="B104" s="1"/>
+      <c r="C104" s="1"/>
+      <c r="D104" s="1"/>
+      <c r="E104" s="1"/>
+      <c r="F104" s="1"/>
+      <c r="G104" s="1"/>
+      <c r="H104" s="1"/>
+      <c r="I104" s="1"/>
+      <c r="J104" s="1"/>
+      <c r="K104" s="1"/>
+      <c r="L104" s="1"/>
+      <c r="M104" s="1"/>
+      <c r="N104" s="1"/>
+      <c r="O104" s="1"/>
+    </row>
+    <row r="105" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A105" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C105" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D105" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E105" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F105" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G105" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H105" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I105" s="1"/>
+      <c r="J105" s="1"/>
+      <c r="K105" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="L105" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="M105" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="N105" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O105" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="106" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A106" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D106" s="2">
+        <v>1</v>
+      </c>
+      <c r="E106" s="3"/>
+      <c r="F106" s="3"/>
+      <c r="G106" s="2"/>
+      <c r="H106" s="2"/>
+      <c r="I106" s="2"/>
+      <c r="J106" s="2"/>
+      <c r="K106" s="3"/>
+      <c r="L106" s="3"/>
+      <c r="M106" s="3"/>
+      <c r="N106" s="3"/>
+      <c r="O106" s="3"/>
+    </row>
+    <row r="107" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A107" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C107" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D107" s="4">
+        <v>1</v>
+      </c>
+      <c r="E107" s="5"/>
+      <c r="F107" s="4"/>
+      <c r="G107" s="4"/>
+      <c r="H107" s="4"/>
+      <c r="I107" s="4"/>
+      <c r="J107" s="4"/>
+      <c r="K107" s="5"/>
+      <c r="L107" s="5"/>
+      <c r="M107" s="4"/>
+      <c r="N107" s="4"/>
+      <c r="O107" s="4"/>
+    </row>
+    <row r="108" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A108" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B108" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C108" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D108" s="2">
+        <v>1</v>
+      </c>
+      <c r="E108" s="3"/>
+      <c r="F108" s="3"/>
+      <c r="G108" s="2"/>
+      <c r="H108" s="2"/>
+      <c r="I108" s="2"/>
+      <c r="J108" s="2"/>
+      <c r="K108" s="3"/>
+      <c r="L108" s="3"/>
+      <c r="M108" s="3"/>
+      <c r="N108" s="3"/>
+      <c r="O108" s="3"/>
+    </row>
+    <row r="109" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A109" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C109" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D109" s="4">
+        <v>1</v>
+      </c>
+      <c r="E109" s="5"/>
+      <c r="F109" s="4"/>
+      <c r="G109" s="4"/>
+      <c r="H109" s="4"/>
+      <c r="I109" s="4"/>
+      <c r="J109" s="4"/>
+      <c r="K109" s="5"/>
+      <c r="L109" s="5"/>
+      <c r="M109" s="4"/>
+      <c r="N109" s="4"/>
+      <c r="O109" s="4"/>
+    </row>
+    <row r="110" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A110" s="1"/>
+      <c r="B110" s="1"/>
+      <c r="C110" s="1"/>
+      <c r="D110" s="1"/>
+      <c r="E110" s="1"/>
+      <c r="F110" s="1"/>
+      <c r="G110" s="1"/>
+      <c r="H110" s="1"/>
+      <c r="I110" s="1"/>
+      <c r="J110" s="1"/>
+      <c r="K110" s="1"/>
+      <c r="L110" s="1"/>
+      <c r="M110" s="1"/>
+      <c r="N110" s="1"/>
+      <c r="O110" s="1"/>
+    </row>
+    <row r="111" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A111" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C111" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D111" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E111" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F111" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G111" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H111" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I111" s="1"/>
+      <c r="J111" s="1"/>
+      <c r="K111" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="L111" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="M111" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="N111" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O111" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="112" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A112" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B112" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C112" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D112" s="2">
+        <v>1</v>
+      </c>
+      <c r="E112" s="3"/>
+      <c r="F112" s="3"/>
+      <c r="G112" s="2"/>
+      <c r="H112" s="2"/>
+      <c r="I112" s="2"/>
+      <c r="J112" s="2"/>
+      <c r="K112" s="3"/>
+      <c r="L112" s="3"/>
+      <c r="M112" s="3"/>
+      <c r="N112" s="3"/>
+      <c r="O112" s="3"/>
+    </row>
+    <row r="113" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A113" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B113" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C113" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D113" s="4">
+        <v>1</v>
+      </c>
+      <c r="E113" s="5"/>
+      <c r="F113" s="4"/>
+      <c r="G113" s="4"/>
+      <c r="H113" s="4"/>
+      <c r="I113" s="4"/>
+      <c r="J113" s="4"/>
+      <c r="K113" s="5"/>
+      <c r="L113" s="5"/>
+      <c r="M113" s="4"/>
+      <c r="N113" s="5"/>
+      <c r="O113" s="4"/>
+    </row>
+    <row r="114" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A114" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B114" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C114" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D114" s="2">
+        <v>1</v>
+      </c>
+      <c r="E114" s="3"/>
+      <c r="F114" s="3"/>
+      <c r="G114" s="2"/>
+      <c r="H114" s="2"/>
+      <c r="I114" s="2"/>
+      <c r="J114" s="2"/>
+      <c r="K114" s="3"/>
+      <c r="L114" s="3"/>
+      <c r="M114" s="3"/>
+      <c r="N114" s="3"/>
+      <c r="O114" s="3"/>
+    </row>
+    <row r="115" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A115" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B115" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C115" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D115" s="4">
+        <v>1</v>
+      </c>
+      <c r="E115" s="5"/>
+      <c r="F115" s="4"/>
+      <c r="G115" s="4"/>
+      <c r="H115" s="4"/>
+      <c r="I115" s="4"/>
+      <c r="J115" s="4"/>
+      <c r="K115" s="5"/>
+      <c r="L115" s="5"/>
+      <c r="M115" s="4"/>
+      <c r="N115" s="5"/>
+      <c r="O115" s="4"/>
+    </row>
+    <row r="116" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A116" s="1"/>
+      <c r="B116" s="1"/>
+      <c r="C116" s="1"/>
+      <c r="D116" s="1"/>
+      <c r="E116" s="1"/>
+      <c r="F116" s="1"/>
+      <c r="G116" s="1"/>
+      <c r="H116" s="1"/>
+      <c r="I116" s="1"/>
+      <c r="J116" s="1"/>
+      <c r="K116" s="1"/>
+      <c r="L116" s="1"/>
+      <c r="M116" s="1"/>
+      <c r="N116" s="1"/>
+      <c r="O116" s="1"/>
+    </row>
+    <row r="117" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A117" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B117" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C117" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D117" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E117" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F117" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G117" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H117" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I117" s="1"/>
+      <c r="J117" s="1"/>
+      <c r="K117" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="L117" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="M117" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="N117" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O117" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="118" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A118" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B118" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C118" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D118" s="2">
+        <v>1</v>
+      </c>
+      <c r="E118" s="3"/>
+      <c r="F118" s="3"/>
+      <c r="G118" s="2"/>
+      <c r="H118" s="2"/>
+      <c r="I118" s="2"/>
+      <c r="J118" s="2"/>
+      <c r="K118" s="3"/>
+      <c r="L118" s="3"/>
+      <c r="M118" s="3"/>
+      <c r="N118" s="3"/>
+      <c r="O118" s="3"/>
+    </row>
+    <row r="119" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A119" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B119" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C119" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D119" s="4">
+        <v>1</v>
+      </c>
+      <c r="E119" s="5"/>
+      <c r="F119" s="4"/>
+      <c r="G119" s="4"/>
+      <c r="H119" s="4"/>
+      <c r="I119" s="4"/>
+      <c r="J119" s="4"/>
+      <c r="K119" s="5"/>
+      <c r="L119" s="5"/>
+      <c r="M119" s="5"/>
+      <c r="N119" s="4"/>
+      <c r="O119" s="4"/>
+    </row>
+    <row r="120" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A120" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B120" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C120" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D120" s="2">
+        <v>1</v>
+      </c>
+      <c r="E120" s="3"/>
+      <c r="F120" s="3"/>
+      <c r="G120" s="2"/>
+      <c r="H120" s="2"/>
+      <c r="I120" s="2"/>
+      <c r="J120" s="2"/>
+      <c r="K120" s="3"/>
+      <c r="L120" s="3"/>
+      <c r="M120" s="3"/>
+      <c r="N120" s="3"/>
+      <c r="O120" s="3"/>
+    </row>
+    <row r="121" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A121" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B121" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C121" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D121" s="4">
+        <v>1</v>
+      </c>
+      <c r="E121" s="5"/>
+      <c r="F121" s="4"/>
+      <c r="G121" s="4"/>
+      <c r="H121" s="4"/>
+      <c r="I121" s="4"/>
+      <c r="J121" s="4"/>
+      <c r="K121" s="5"/>
+      <c r="L121" s="5"/>
+      <c r="M121" s="4"/>
+      <c r="N121" s="4"/>
+      <c r="O121" s="4"/>
+    </row>
+    <row r="122" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A122" s="1"/>
+      <c r="B122" s="1"/>
+      <c r="C122" s="1"/>
+      <c r="D122" s="1"/>
+      <c r="E122" s="1"/>
+      <c r="F122" s="1"/>
+      <c r="G122" s="1"/>
+      <c r="H122" s="1"/>
+      <c r="I122" s="1"/>
+      <c r="J122" s="1"/>
+      <c r="K122" s="1"/>
+      <c r="L122" s="1"/>
+      <c r="M122" s="1"/>
+      <c r="N122" s="1"/>
+      <c r="O122" s="1"/>
+    </row>
+    <row r="123" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A123" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B123" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C123" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D123" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E123" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F123" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G123" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H123" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I123" s="1"/>
+      <c r="J123" s="1"/>
+      <c r="K123" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="L123" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="M123" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="N123" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O123" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="124" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A124" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B124" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C124" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D124" s="2">
+        <v>1</v>
+      </c>
+      <c r="E124" s="3"/>
+      <c r="F124" s="3"/>
+      <c r="G124" s="2"/>
+      <c r="H124" s="2"/>
+      <c r="I124" s="2"/>
+      <c r="J124" s="2"/>
+      <c r="K124" s="3"/>
+      <c r="L124" s="3"/>
+      <c r="M124" s="3"/>
+      <c r="N124" s="3"/>
+      <c r="O124" s="3"/>
+    </row>
+    <row r="125" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A125" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B125" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C125" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D125" s="4">
+        <v>1</v>
+      </c>
+      <c r="E125" s="5"/>
+      <c r="F125" s="5"/>
+      <c r="G125" s="4"/>
+      <c r="H125" s="4"/>
+      <c r="I125" s="4"/>
+      <c r="J125" s="4"/>
+      <c r="K125" s="5"/>
+      <c r="L125" s="5"/>
+      <c r="M125" s="4"/>
+      <c r="N125" s="5"/>
+      <c r="O125" s="5"/>
+    </row>
+    <row r="126" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A126" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B126" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C126" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D126" s="2">
+        <v>1</v>
+      </c>
+      <c r="E126" s="3"/>
+      <c r="F126" s="3"/>
+      <c r="G126" s="2"/>
+      <c r="H126" s="2"/>
+      <c r="I126" s="2"/>
+      <c r="J126" s="2"/>
+      <c r="K126" s="3"/>
+      <c r="L126" s="3"/>
+      <c r="M126" s="3"/>
+      <c r="N126" s="3"/>
+      <c r="O126" s="3"/>
+    </row>
+    <row r="127" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A127" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B127" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C127" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D127" s="4">
+        <v>1</v>
+      </c>
+      <c r="E127" s="5"/>
+      <c r="F127" s="5"/>
+      <c r="G127" s="4"/>
+      <c r="H127" s="4"/>
+      <c r="I127" s="4"/>
+      <c r="J127" s="4"/>
+      <c r="K127" s="5"/>
+      <c r="L127" s="5"/>
+      <c r="M127" s="4"/>
+      <c r="N127" s="5"/>
+      <c r="O127" s="5"/>
+    </row>
+    <row r="135" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A135">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="137" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A137" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B137" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C137" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D137" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E137" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F137" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G137" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H137" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I137" s="1"/>
+      <c r="J137" s="1"/>
+      <c r="K137" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="L137" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="M137" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="N137" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O137" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="138" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A138" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B138" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C138" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D138" s="2">
+        <v>1</v>
+      </c>
+      <c r="E138" s="3"/>
+      <c r="F138" s="3"/>
+      <c r="G138" s="2"/>
+      <c r="H138" s="2"/>
+      <c r="I138" s="2"/>
+      <c r="J138" s="2"/>
+      <c r="K138" s="3"/>
+      <c r="L138" s="3"/>
+      <c r="M138" s="3"/>
+      <c r="N138" s="3"/>
+      <c r="O138" s="3"/>
+    </row>
+    <row r="139" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A139" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B139" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C139" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D139" s="4">
+        <v>1</v>
+      </c>
+      <c r="E139" s="5"/>
+      <c r="F139" s="4"/>
+      <c r="G139" s="4"/>
+      <c r="H139" s="4"/>
+      <c r="I139" s="4"/>
+      <c r="J139" s="4"/>
+      <c r="K139" s="5"/>
+      <c r="L139" s="5"/>
+      <c r="M139" s="4"/>
+      <c r="N139" s="4"/>
+      <c r="O139" s="4"/>
+    </row>
+    <row r="140" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A140" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B140" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C140" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D140" s="2">
+        <v>1</v>
+      </c>
+      <c r="E140" s="3"/>
+      <c r="F140" s="3"/>
+      <c r="G140" s="2"/>
+      <c r="H140" s="2"/>
+      <c r="I140" s="2"/>
+      <c r="J140" s="2"/>
+      <c r="K140" s="3"/>
+      <c r="L140" s="3"/>
+      <c r="M140" s="3"/>
+      <c r="N140" s="3"/>
+      <c r="O140" s="3"/>
+    </row>
+    <row r="141" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A141" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B141" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C141" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D141" s="4">
+        <v>1</v>
+      </c>
+      <c r="E141" s="5"/>
+      <c r="F141" s="4"/>
+      <c r="G141" s="4"/>
+      <c r="H141" s="4"/>
+      <c r="I141" s="4"/>
+      <c r="J141" s="4"/>
+      <c r="K141" s="5"/>
+      <c r="L141" s="5"/>
+      <c r="M141" s="4"/>
+      <c r="N141" s="4"/>
+      <c r="O141" s="4"/>
+    </row>
+    <row r="142" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A142" s="1"/>
+      <c r="B142" s="1"/>
+      <c r="C142" s="1"/>
+      <c r="D142" s="1"/>
+      <c r="E142" s="1"/>
+      <c r="F142" s="1"/>
+      <c r="G142" s="1"/>
+      <c r="H142" s="1"/>
+      <c r="I142" s="1"/>
+      <c r="J142" s="1"/>
+      <c r="K142" s="1"/>
+      <c r="L142" s="1"/>
+      <c r="M142" s="1"/>
+      <c r="N142" s="1"/>
+      <c r="O142" s="1"/>
+    </row>
+    <row r="143" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A143" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B143" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C143" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D143" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E143" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F143" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G143" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H143" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I143" s="1"/>
+      <c r="J143" s="1"/>
+      <c r="K143" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="L143" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="M143" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="N143" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O143" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="144" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A144" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B144" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C144" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D144" s="2">
+        <v>1</v>
+      </c>
+      <c r="E144" s="3"/>
+      <c r="F144" s="3"/>
+      <c r="G144" s="2"/>
+      <c r="H144" s="2"/>
+      <c r="I144" s="2"/>
+      <c r="J144" s="2"/>
+      <c r="K144" s="3"/>
+      <c r="L144" s="3"/>
+      <c r="M144" s="3"/>
+      <c r="N144" s="3"/>
+      <c r="O144" s="3"/>
+    </row>
+    <row r="145" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A145" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B145" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C145" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D145" s="4">
+        <v>1</v>
+      </c>
+      <c r="E145" s="5"/>
+      <c r="F145" s="5"/>
+      <c r="G145" s="4"/>
+      <c r="H145" s="4"/>
+      <c r="I145" s="4"/>
+      <c r="J145" s="4"/>
+      <c r="K145" s="5"/>
+      <c r="L145" s="5"/>
+      <c r="M145" s="4"/>
+      <c r="N145" s="5"/>
+      <c r="O145" s="5"/>
+    </row>
+    <row r="146" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A146" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B146" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C146" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D146" s="2">
+        <v>1</v>
+      </c>
+      <c r="E146" s="3"/>
+      <c r="F146" s="3"/>
+      <c r="G146" s="2"/>
+      <c r="H146" s="2"/>
+      <c r="I146" s="2"/>
+      <c r="J146" s="2"/>
+      <c r="K146" s="3"/>
+      <c r="L146" s="3"/>
+      <c r="M146" s="3"/>
+      <c r="N146" s="3"/>
+      <c r="O146" s="3"/>
+    </row>
+    <row r="147" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A147" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B147" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C147" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D147" s="4">
+        <v>1</v>
+      </c>
+      <c r="E147" s="5"/>
+      <c r="F147" s="4"/>
+      <c r="G147" s="4"/>
+      <c r="H147" s="4"/>
+      <c r="I147" s="4"/>
+      <c r="J147" s="4"/>
+      <c r="K147" s="5"/>
+      <c r="L147" s="5"/>
+      <c r="M147" s="5"/>
+      <c r="N147" s="4"/>
+      <c r="O147" s="4"/>
+    </row>
+    <row r="148" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A148" s="1"/>
+      <c r="B148" s="1"/>
+      <c r="C148" s="1"/>
+      <c r="D148" s="1"/>
+      <c r="E148" s="1"/>
+      <c r="F148" s="1"/>
+      <c r="G148" s="1"/>
+      <c r="H148" s="1"/>
+      <c r="I148" s="1"/>
+      <c r="J148" s="1"/>
+      <c r="K148" s="1"/>
+      <c r="L148" s="1"/>
+      <c r="M148" s="1"/>
+      <c r="N148" s="1"/>
+      <c r="O148" s="1"/>
+    </row>
+    <row r="149" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A149" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B149" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C149" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D149" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E149" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F149" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G149" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H149" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I149" s="1"/>
+      <c r="J149" s="1"/>
+      <c r="K149" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="L149" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="M149" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="N149" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O149" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="150" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A150" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B150" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C150" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D150" s="2">
+        <v>1</v>
+      </c>
+      <c r="E150" s="3"/>
+      <c r="F150" s="3"/>
+      <c r="G150" s="2"/>
+      <c r="H150" s="2"/>
+      <c r="I150" s="2"/>
+      <c r="J150" s="2"/>
+      <c r="K150" s="3"/>
+      <c r="L150" s="3"/>
+      <c r="M150" s="2"/>
+      <c r="N150" s="3"/>
+      <c r="O150" s="3"/>
+    </row>
+    <row r="151" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A151" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B151" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C151" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D151" s="4">
+        <v>1</v>
+      </c>
+      <c r="E151" s="5"/>
+      <c r="F151" s="4"/>
+      <c r="G151" s="4"/>
+      <c r="H151" s="4"/>
+      <c r="I151" s="4"/>
+      <c r="J151" s="4"/>
+      <c r="K151" s="5"/>
+      <c r="L151" s="5"/>
+      <c r="M151" s="4"/>
+      <c r="N151" s="4"/>
+      <c r="O151" s="4"/>
+    </row>
+    <row r="152" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A152" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B152" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C152" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D152" s="2">
+        <v>1</v>
+      </c>
+      <c r="E152" s="3"/>
+      <c r="F152" s="3"/>
+      <c r="G152" s="2"/>
+      <c r="H152" s="2"/>
+      <c r="I152" s="2"/>
+      <c r="J152" s="2"/>
+      <c r="K152" s="3"/>
+      <c r="L152" s="3"/>
+      <c r="M152" s="3"/>
+      <c r="N152" s="3"/>
+      <c r="O152" s="3"/>
+    </row>
+    <row r="153" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A153" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B153" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C153" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D153" s="4">
+        <v>1</v>
+      </c>
+      <c r="E153" s="5">
+        <v>12101</v>
+      </c>
+      <c r="F153" s="5">
+        <v>1031</v>
+      </c>
+      <c r="G153" s="4">
+        <v>96</v>
+      </c>
+      <c r="H153" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="I153" s="4"/>
+      <c r="J153" s="4"/>
+      <c r="K153" s="5">
+        <v>12833</v>
+      </c>
+      <c r="L153" s="5">
+        <v>11989</v>
+      </c>
+      <c r="M153" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="N153" s="5">
+        <v>1039</v>
+      </c>
+      <c r="O153" s="5">
+        <v>1027</v>
+      </c>
+    </row>
+    <row r="154" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A154" s="1"/>
+      <c r="B154" s="1"/>
+      <c r="C154" s="1"/>
+      <c r="D154" s="1"/>
+      <c r="E154" s="1"/>
+      <c r="F154" s="1"/>
+      <c r="G154" s="1"/>
+      <c r="H154" s="1"/>
+      <c r="I154" s="1"/>
+      <c r="J154" s="1"/>
+      <c r="K154" s="1"/>
+      <c r="L154" s="1"/>
+      <c r="M154" s="1"/>
+      <c r="N154" s="1"/>
+      <c r="O154" s="1"/>
+    </row>
+    <row r="155" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A155" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B155" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C155" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D155" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E155" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F155" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G155" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H155" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I155" s="1"/>
+      <c r="J155" s="1"/>
+      <c r="K155" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="L155" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="M155" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="N155" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O155" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="156" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A156" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B156" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C156" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D156" s="2">
+        <v>1</v>
+      </c>
+      <c r="E156" s="3"/>
+      <c r="F156" s="3"/>
+      <c r="G156" s="2"/>
+      <c r="H156" s="2"/>
+      <c r="I156" s="2"/>
+      <c r="J156" s="2"/>
+      <c r="K156" s="3"/>
+      <c r="L156" s="3"/>
+      <c r="M156" s="3"/>
+      <c r="N156" s="3"/>
+      <c r="O156" s="3"/>
+    </row>
+    <row r="157" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A157" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B157" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C157" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D157" s="4">
+        <v>1</v>
+      </c>
+      <c r="E157" s="5"/>
+      <c r="F157" s="4"/>
+      <c r="G157" s="4"/>
+      <c r="H157" s="4"/>
+      <c r="I157" s="4"/>
+      <c r="J157" s="4"/>
+      <c r="K157" s="5"/>
+      <c r="L157" s="5"/>
+      <c r="M157" s="4"/>
+      <c r="N157" s="4"/>
+      <c r="O157" s="4"/>
+    </row>
+    <row r="158" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A158" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B158" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C158" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D158" s="2">
+        <v>1</v>
+      </c>
+      <c r="E158" s="3"/>
+      <c r="F158" s="3"/>
+      <c r="G158" s="2"/>
+      <c r="H158" s="2"/>
+      <c r="I158" s="2"/>
+      <c r="J158" s="2"/>
+      <c r="K158" s="3"/>
+      <c r="L158" s="3"/>
+      <c r="M158" s="3"/>
+      <c r="N158" s="3"/>
+      <c r="O158" s="3"/>
+    </row>
+    <row r="159" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A159" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B159" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C159" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D159" s="4">
+        <v>1</v>
+      </c>
+      <c r="E159" s="5"/>
+      <c r="F159" s="5"/>
+      <c r="G159" s="4"/>
+      <c r="H159" s="4"/>
+      <c r="I159" s="4"/>
+      <c r="J159" s="4"/>
+      <c r="K159" s="5"/>
+      <c r="L159" s="5"/>
+      <c r="M159" s="4"/>
+      <c r="N159" s="5"/>
+      <c r="O159" s="5"/>
+    </row>
+    <row r="160" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A160" s="1"/>
+      <c r="B160" s="1"/>
+      <c r="C160" s="1"/>
+      <c r="D160" s="1"/>
+      <c r="E160" s="1"/>
+      <c r="F160" s="1"/>
+      <c r="G160" s="1"/>
+      <c r="H160" s="1"/>
+      <c r="I160" s="1"/>
+      <c r="J160" s="1"/>
+      <c r="K160" s="1"/>
+      <c r="L160" s="1"/>
+      <c r="M160" s="1"/>
+      <c r="N160" s="1"/>
+      <c r="O160" s="1"/>
+    </row>
+    <row r="161" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A161" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B161" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C161" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D161" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E161" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F161" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G161" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H161" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I161" s="1"/>
+      <c r="J161" s="1"/>
+      <c r="K161" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="L161" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="M161" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="N161" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O161" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="162" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A162" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B162" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C162" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D162" s="2">
+        <v>1</v>
+      </c>
+      <c r="E162" s="3"/>
+      <c r="F162" s="3"/>
+      <c r="G162" s="2"/>
+      <c r="H162" s="2"/>
+      <c r="I162" s="2"/>
+      <c r="J162" s="2"/>
+      <c r="K162" s="3"/>
+      <c r="L162" s="3"/>
+      <c r="M162" s="3"/>
+      <c r="N162" s="3"/>
+      <c r="O162" s="3"/>
+    </row>
+    <row r="163" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A163" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B163" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C163" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D163" s="4">
+        <v>1</v>
+      </c>
+      <c r="E163" s="5"/>
+      <c r="F163" s="5"/>
+      <c r="G163" s="4"/>
+      <c r="H163" s="4"/>
+      <c r="I163" s="4"/>
+      <c r="J163" s="4"/>
+      <c r="K163" s="5"/>
+      <c r="L163" s="5"/>
+      <c r="M163" s="5"/>
+      <c r="N163" s="5"/>
+      <c r="O163" s="5"/>
+    </row>
+    <row r="164" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A164" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B164" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C164" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D164" s="2">
+        <v>1</v>
+      </c>
+      <c r="E164" s="3"/>
+      <c r="F164" s="3"/>
+      <c r="G164" s="2"/>
+      <c r="H164" s="2"/>
+      <c r="I164" s="2"/>
+      <c r="J164" s="2"/>
+      <c r="K164" s="3"/>
+      <c r="L164" s="3"/>
+      <c r="M164" s="3"/>
+      <c r="N164" s="3"/>
+      <c r="O164" s="3"/>
+    </row>
+    <row r="165" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A165" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B165" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C165" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D165" s="4">
+        <v>1</v>
+      </c>
+      <c r="E165" s="5"/>
+      <c r="F165" s="5"/>
+      <c r="G165" s="4"/>
+      <c r="H165" s="4"/>
+      <c r="I165" s="4"/>
+      <c r="J165" s="4"/>
+      <c r="K165" s="5"/>
+      <c r="L165" s="5"/>
+      <c r="M165" s="4"/>
+      <c r="N165" s="5"/>
+      <c r="O165" s="5"/>
+    </row>
+    <row r="166" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A166" s="1"/>
+      <c r="B166" s="1"/>
+      <c r="C166" s="1"/>
+      <c r="D166" s="1"/>
+      <c r="E166" s="1"/>
+      <c r="F166" s="1"/>
+      <c r="G166" s="1"/>
+      <c r="H166" s="1"/>
+      <c r="I166" s="1"/>
+      <c r="J166" s="1"/>
+      <c r="K166" s="1"/>
+      <c r="L166" s="1"/>
+      <c r="M166" s="1"/>
+      <c r="N166" s="1"/>
+      <c r="O166" s="1"/>
+    </row>
+    <row r="183" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A183" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="184" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A184">
+        <v>2024</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
updated runtimes for partB
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vanessa\Documents\Uni\Bachelor-Thesis\BachelorThesis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/21c1a4ced64a9754/Documents/Uni/Bachelor Thesis/BachelorThesis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30350997-3BBF-49AB-916C-212AA2CBCFFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="287" documentId="13_ncr:1_{30350997-3BBF-49AB-916C-212AA2CBCFFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A8736EF-0517-47FB-A85B-0A84D8E72BDF}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{2A4234DB-3A22-4351-83C3-53CA1AE1142A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{2A4234DB-3A22-4351-83C3-53CA1AE1142A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="677" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="734" uniqueCount="141">
   <si>
     <t>Benchmarking results LLMs</t>
   </si>
@@ -342,6 +342,123 @@
   </si>
   <si>
     <t>Part B</t>
+  </si>
+  <si>
+    <t>0.570</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.405</t>
+  </si>
+  <si>
+    <t>0.562</t>
+  </si>
+  <si>
+    <t>0.148</t>
+  </si>
+  <si>
+    <t>0.967</t>
+  </si>
+  <si>
+    <t>0.969</t>
+  </si>
+  <si>
+    <t>0.228</t>
+  </si>
+  <si>
+    <t>0.924</t>
+  </si>
+  <si>
+    <t>0.922</t>
+  </si>
+  <si>
+    <t>0.926</t>
+  </si>
+  <si>
+    <t>0.141</t>
+  </si>
+  <si>
+    <t>0.223</t>
+  </si>
+  <si>
+    <t>0.963</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.965 </t>
+  </si>
+  <si>
+    <t>0.410</t>
+  </si>
+  <si>
+    <t>0.224</t>
+  </si>
+  <si>
+    <t>0.423</t>
+  </si>
+  <si>
+    <t>0.143</t>
+  </si>
+  <si>
+    <t>0.921</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.918 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.922 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.203 </t>
+  </si>
+  <si>
+    <t>0.192</t>
+  </si>
+  <si>
+    <t>0.943</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.202</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.565</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.926</t>
+  </si>
+  <si>
+    <t>0.543</t>
+  </si>
+  <si>
+    <t>0.037</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.648</t>
+  </si>
+  <si>
+    <t>0.024</t>
+  </si>
+  <si>
+    <t>0.839</t>
+  </si>
+  <si>
+    <t>0.442</t>
+  </si>
+  <si>
+    <t>0.285</t>
+  </si>
+  <si>
+    <t>0.915</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.910</t>
+  </si>
+  <si>
+    <t>0.939</t>
+  </si>
+  <si>
+    <t>0.046</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.191 </t>
   </si>
 </sst>
 </file>
@@ -406,7 +523,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -426,6 +543,7 @@
     <xf numFmtId="164" fontId="2" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Bad" xfId="2" builtinId="27"/>
@@ -763,19 +881,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9626A942-19B5-4B39-BBE2-849051787A6F}">
   <dimension ref="A1:O184"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="5" max="5" width="15.28515625" customWidth="1"/>
-    <col min="6" max="6" width="15.140625" customWidth="1"/>
-    <col min="8" max="8" width="50.140625" customWidth="1"/>
-    <col min="11" max="11" width="13.85546875" customWidth="1"/>
-    <col min="12" max="12" width="12.85546875" customWidth="1"/>
-    <col min="14" max="14" width="14.42578125" customWidth="1"/>
-    <col min="15" max="15" width="14.85546875" customWidth="1"/>
-    <col min="16" max="16" width="13.7109375" customWidth="1"/>
+    <col min="5" max="5" width="15.26953125" customWidth="1"/>
+    <col min="6" max="6" width="15.1796875" customWidth="1"/>
+    <col min="8" max="8" width="50.1796875" customWidth="1"/>
+    <col min="11" max="11" width="13.81640625" customWidth="1"/>
+    <col min="12" max="12" width="12.81640625" customWidth="1"/>
+    <col min="14" max="14" width="14.453125" customWidth="1"/>
+    <col min="15" max="15" width="14.81640625" customWidth="1"/>
+    <col min="16" max="16" width="13.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -786,12 +904,12 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>2024</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
@@ -834,7 +952,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
@@ -877,7 +995,7 @@
         <v>7004</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
         <v>9</v>
       </c>
@@ -920,7 +1038,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>9</v>
       </c>
@@ -963,7 +1081,7 @@
         <v>7328</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
         <v>9</v>
       </c>
@@ -1006,7 +1124,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -1023,7 +1141,7 @@
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>1</v>
       </c>
@@ -1066,7 +1184,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>23</v>
       </c>
@@ -1109,7 +1227,7 @@
         <v>6961</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A14" s="4" t="s">
         <v>23</v>
       </c>
@@ -1152,7 +1270,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -1195,7 +1313,7 @@
         <v>7055</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
         <v>23</v>
       </c>
@@ -1238,7 +1356,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -1255,7 +1373,7 @@
       <c r="N17" s="1"/>
       <c r="O17" s="1"/>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>1</v>
       </c>
@@ -1298,7 +1416,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>24</v>
       </c>
@@ -1341,7 +1459,7 @@
         <v>7141</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A20" s="4" t="s">
         <v>24</v>
       </c>
@@ -1384,7 +1502,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>24</v>
       </c>
@@ -1427,7 +1545,7 @@
         <v>7117</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A22" s="4" t="s">
         <v>24</v>
       </c>
@@ -1470,7 +1588,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -1487,7 +1605,7 @@
       <c r="N23" s="1"/>
       <c r="O23" s="1"/>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>1</v>
       </c>
@@ -1530,7 +1648,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>25</v>
       </c>
@@ -1573,7 +1691,7 @@
         <v>7172</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A26" s="4" t="s">
         <v>25</v>
       </c>
@@ -1616,7 +1734,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>25</v>
       </c>
@@ -1659,7 +1777,7 @@
         <v>7602</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A28" s="4" t="s">
         <v>25</v>
       </c>
@@ -1702,7 +1820,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -1719,7 +1837,7 @@
       <c r="N29" s="1"/>
       <c r="O29" s="1"/>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>1</v>
       </c>
@@ -1762,7 +1880,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>26</v>
       </c>
@@ -1805,7 +1923,7 @@
         <v>7078</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A32" s="4" t="s">
         <v>26</v>
       </c>
@@ -1848,7 +1966,7 @@
         <v>1031</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>26</v>
       </c>
@@ -1891,7 +2009,7 @@
         <v>7121</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A34" s="4" t="s">
         <v>26</v>
       </c>
@@ -1934,7 +2052,7 @@
         <v>1039</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
@@ -1951,7 +2069,7 @@
       <c r="N35" s="1"/>
       <c r="O35" s="1"/>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>1</v>
       </c>
@@ -1994,7 +2112,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>27</v>
       </c>
@@ -2037,7 +2155,7 @@
         <v>7078</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A38" s="4" t="s">
         <v>27</v>
       </c>
@@ -2080,7 +2198,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>27</v>
       </c>
@@ -2123,7 +2241,7 @@
         <v>7074</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A40" s="4" t="s">
         <v>27</v>
       </c>
@@ -2166,12 +2284,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>2025</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>1</v>
       </c>
@@ -2214,7 +2332,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
         <v>9</v>
       </c>
@@ -2257,7 +2375,7 @@
         <v>6934</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A52" s="4" t="s">
         <v>9</v>
       </c>
@@ -2300,7 +2418,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
         <v>9</v>
       </c>
@@ -2343,7 +2461,7 @@
         <v>7180</v>
       </c>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A54" s="4" t="s">
         <v>9</v>
       </c>
@@ -2386,7 +2504,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A55" s="1"/>
       <c r="B55" s="1"/>
       <c r="C55" s="1"/>
@@ -2403,7 +2521,7 @@
       <c r="N55" s="1"/>
       <c r="O55" s="1"/>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>1</v>
       </c>
@@ -2446,7 +2564,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
         <v>23</v>
       </c>
@@ -2489,7 +2607,7 @@
         <v>7012</v>
       </c>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A58" s="4" t="s">
         <v>23</v>
       </c>
@@ -2532,7 +2650,7 @@
         <v>2004</v>
       </c>
     </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
         <v>23</v>
       </c>
@@ -2575,7 +2693,7 @@
         <v>10863</v>
       </c>
     </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A60" s="4" t="s">
         <v>23</v>
       </c>
@@ -2618,7 +2736,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A61" s="1"/>
       <c r="B61" s="1"/>
       <c r="C61" s="1"/>
@@ -2635,7 +2753,7 @@
       <c r="N61" s="1"/>
       <c r="O61" s="1"/>
     </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>1</v>
       </c>
@@ -2678,7 +2796,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A63" s="2" t="s">
         <v>53</v>
       </c>
@@ -2721,7 +2839,7 @@
         <v>7102</v>
       </c>
     </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A64" s="4" t="s">
         <v>53</v>
       </c>
@@ -2764,7 +2882,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A65" s="2" t="s">
         <v>53</v>
       </c>
@@ -2807,7 +2925,7 @@
         <v>7191</v>
       </c>
     </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A66" s="4" t="s">
         <v>53</v>
       </c>
@@ -2850,7 +2968,7 @@
         <v>1027</v>
       </c>
     </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A67" s="1"/>
       <c r="B67" s="1"/>
       <c r="C67" s="1"/>
@@ -2867,7 +2985,7 @@
       <c r="N67" s="1"/>
       <c r="O67" s="1"/>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
         <v>1</v>
       </c>
@@ -2910,7 +3028,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A69" s="2" t="s">
         <v>54</v>
       </c>
@@ -2953,7 +3071,7 @@
         <v>6980</v>
       </c>
     </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A70" s="4" t="s">
         <v>54</v>
       </c>
@@ -2996,7 +3114,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A71" s="2" t="s">
         <v>54</v>
       </c>
@@ -3039,7 +3157,7 @@
         <v>7938</v>
       </c>
     </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A72" s="4" t="s">
         <v>54</v>
       </c>
@@ -3082,7 +3200,7 @@
         <v>1047</v>
       </c>
     </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A73" s="1"/>
       <c r="B73" s="1"/>
       <c r="C73" s="1"/>
@@ -3099,7 +3217,7 @@
       <c r="N73" s="1"/>
       <c r="O73" s="1"/>
     </row>
-    <row r="74" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A74" s="1" t="s">
         <v>1</v>
       </c>
@@ -3142,7 +3260,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A75" s="2" t="s">
         <v>55</v>
       </c>
@@ -3185,7 +3303,7 @@
         <v>7105</v>
       </c>
     </row>
-    <row r="76" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A76" s="4" t="s">
         <v>55</v>
       </c>
@@ -3228,7 +3346,7 @@
         <v>1152</v>
       </c>
     </row>
-    <row r="77" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A77" s="2" t="s">
         <v>55</v>
       </c>
@@ -3271,7 +3389,7 @@
         <v>7098</v>
       </c>
     </row>
-    <row r="78" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A78" s="4" t="s">
         <v>55</v>
       </c>
@@ -3314,7 +3432,7 @@
         <v>1148</v>
       </c>
     </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
       <c r="C79" s="1"/>
@@ -3331,7 +3449,7 @@
       <c r="N79" s="1"/>
       <c r="O79" s="1"/>
     </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A80" s="1" t="s">
         <v>1</v>
       </c>
@@ -3374,7 +3492,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="81" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A81" s="2" t="s">
         <v>24</v>
       </c>
@@ -3417,7 +3535,7 @@
         <v>7156</v>
       </c>
     </row>
-    <row r="82" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A82" s="4" t="s">
         <v>24</v>
       </c>
@@ -3460,7 +3578,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="83" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A83" s="2" t="s">
         <v>24</v>
       </c>
@@ -3503,7 +3621,7 @@
         <v>7160</v>
       </c>
     </row>
-    <row r="84" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A84" s="4" t="s">
         <v>24</v>
       </c>
@@ -3546,17 +3664,17 @@
         <v>78</v>
       </c>
     </row>
-    <row r="96" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="97" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A97">
         <v>2024</v>
       </c>
     </row>
-    <row r="99" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A99" s="1" t="s">
         <v>1</v>
       </c>
@@ -3599,7 +3717,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="100" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A100" s="2" t="s">
         <v>9</v>
       </c>
@@ -3612,19 +3730,33 @@
       <c r="D100" s="2">
         <v>1</v>
       </c>
-      <c r="E100" s="3"/>
-      <c r="F100" s="3"/>
+      <c r="E100" s="3">
+        <v>32326</v>
+      </c>
+      <c r="F100" s="3">
+        <v>6984</v>
+      </c>
       <c r="G100" s="2"/>
       <c r="H100" s="2"/>
       <c r="I100" s="2"/>
       <c r="J100" s="2"/>
-      <c r="K100" s="3"/>
-      <c r="L100" s="3"/>
-      <c r="M100" s="3"/>
-      <c r="N100" s="3"/>
-      <c r="O100" s="3"/>
-    </row>
-    <row r="101" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K100" s="3">
+        <v>33257</v>
+      </c>
+      <c r="L100" s="3">
+        <v>31387</v>
+      </c>
+      <c r="M100" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="N100" s="3">
+        <v>6988</v>
+      </c>
+      <c r="O100" s="3">
+        <v>6980</v>
+      </c>
+    </row>
+    <row r="101" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A101" s="4" t="s">
         <v>9</v>
       </c>
@@ -3637,19 +3769,33 @@
       <c r="D101" s="4">
         <v>1</v>
       </c>
-      <c r="E101" s="5"/>
-      <c r="F101" s="6"/>
+      <c r="E101" s="5">
+        <v>11954</v>
+      </c>
+      <c r="F101" s="6" t="s">
+        <v>106</v>
+      </c>
       <c r="G101" s="4"/>
       <c r="H101" s="4"/>
       <c r="I101" s="4"/>
       <c r="J101" s="4"/>
-      <c r="K101" s="5"/>
-      <c r="L101" s="5"/>
-      <c r="M101" s="4"/>
-      <c r="N101" s="4"/>
-      <c r="O101" s="4"/>
-    </row>
-    <row r="102" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K101" s="5">
+        <v>12020</v>
+      </c>
+      <c r="L101" s="5">
+        <v>11532</v>
+      </c>
+      <c r="M101" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="N101" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="O101" s="4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="102" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A102" s="2" t="s">
         <v>9</v>
       </c>
@@ -3662,19 +3808,33 @@
       <c r="D102" s="2">
         <v>1</v>
       </c>
-      <c r="E102" s="3"/>
-      <c r="F102" s="3"/>
+      <c r="E102" s="3">
+        <v>34248</v>
+      </c>
+      <c r="F102" s="3">
+        <v>7305</v>
+      </c>
       <c r="G102" s="2"/>
       <c r="H102" s="2"/>
       <c r="I102" s="2"/>
       <c r="J102" s="2"/>
-      <c r="K102" s="3"/>
-      <c r="L102" s="3"/>
-      <c r="M102" s="3"/>
-      <c r="N102" s="3"/>
-      <c r="O102" s="3"/>
-    </row>
-    <row r="103" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K102" s="3">
+        <v>40697</v>
+      </c>
+      <c r="L102" s="3">
+        <v>31461</v>
+      </c>
+      <c r="M102" s="3">
+        <v>3572</v>
+      </c>
+      <c r="N102" s="3">
+        <v>7309</v>
+      </c>
+      <c r="O102" s="3">
+        <v>7301</v>
+      </c>
+    </row>
+    <row r="103" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A103" s="4" t="s">
         <v>9</v>
       </c>
@@ -3687,19 +3847,33 @@
       <c r="D103" s="4">
         <v>1</v>
       </c>
-      <c r="E103" s="5"/>
-      <c r="F103" s="4"/>
+      <c r="E103" s="5">
+        <v>11970</v>
+      </c>
+      <c r="F103" s="4" t="s">
+        <v>114</v>
+      </c>
       <c r="G103" s="4"/>
       <c r="H103" s="4"/>
       <c r="I103" s="4"/>
       <c r="J103" s="4"/>
-      <c r="K103" s="5"/>
-      <c r="L103" s="5"/>
-      <c r="M103" s="4"/>
-      <c r="N103" s="4"/>
-      <c r="O103" s="4"/>
-    </row>
-    <row r="104" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K103" s="5">
+        <v>13009</v>
+      </c>
+      <c r="L103" s="5">
+        <v>11529</v>
+      </c>
+      <c r="M103" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="N103" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="O103" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="104" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A104" s="1"/>
       <c r="B104" s="1"/>
       <c r="C104" s="1"/>
@@ -3716,7 +3890,7 @@
       <c r="N104" s="1"/>
       <c r="O104" s="1"/>
     </row>
-    <row r="105" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A105" s="1" t="s">
         <v>1</v>
       </c>
@@ -3759,7 +3933,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="106" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A106" s="2" t="s">
         <v>23</v>
       </c>
@@ -3772,19 +3946,33 @@
       <c r="D106" s="2">
         <v>1</v>
       </c>
-      <c r="E106" s="3"/>
-      <c r="F106" s="3"/>
+      <c r="E106" s="3">
+        <v>33799</v>
+      </c>
+      <c r="F106" s="3">
+        <v>6973</v>
+      </c>
       <c r="G106" s="2"/>
       <c r="H106" s="2"/>
       <c r="I106" s="2"/>
       <c r="J106" s="2"/>
-      <c r="K106" s="3"/>
-      <c r="L106" s="3"/>
-      <c r="M106" s="3"/>
-      <c r="N106" s="3"/>
-      <c r="O106" s="3"/>
-    </row>
-    <row r="107" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K106" s="3">
+        <v>34659</v>
+      </c>
+      <c r="L106" s="3">
+        <v>33237</v>
+      </c>
+      <c r="M106" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="N106" s="3">
+        <v>6977</v>
+      </c>
+      <c r="O106" s="3">
+        <v>6969</v>
+      </c>
+    </row>
+    <row r="107" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A107" s="4" t="s">
         <v>23</v>
       </c>
@@ -3797,19 +3985,33 @@
       <c r="D107" s="4">
         <v>1</v>
       </c>
-      <c r="E107" s="5"/>
-      <c r="F107" s="4"/>
+      <c r="E107" s="5">
+        <v>11986</v>
+      </c>
+      <c r="F107" s="4" t="s">
+        <v>109</v>
+      </c>
       <c r="G107" s="4"/>
       <c r="H107" s="4"/>
       <c r="I107" s="4"/>
       <c r="J107" s="4"/>
-      <c r="K107" s="5"/>
-      <c r="L107" s="5"/>
-      <c r="M107" s="4"/>
-      <c r="N107" s="4"/>
-      <c r="O107" s="4"/>
-    </row>
-    <row r="108" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K107" s="5">
+        <v>12500</v>
+      </c>
+      <c r="L107" s="5">
+        <v>11602</v>
+      </c>
+      <c r="M107" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="N107" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="O107" s="4" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="108" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A108" s="2" t="s">
         <v>23</v>
       </c>
@@ -3822,19 +4024,33 @@
       <c r="D108" s="2">
         <v>1</v>
       </c>
-      <c r="E108" s="3"/>
-      <c r="F108" s="3"/>
+      <c r="E108" s="3">
+        <v>37333</v>
+      </c>
+      <c r="F108" s="3">
+        <v>7034</v>
+      </c>
       <c r="G108" s="2"/>
       <c r="H108" s="2"/>
       <c r="I108" s="2"/>
       <c r="J108" s="2"/>
-      <c r="K108" s="3"/>
-      <c r="L108" s="3"/>
-      <c r="M108" s="3"/>
-      <c r="N108" s="3"/>
-      <c r="O108" s="3"/>
-    </row>
-    <row r="109" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K108" s="3">
+        <v>37828</v>
+      </c>
+      <c r="L108" s="3">
+        <v>37106</v>
+      </c>
+      <c r="M108" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="N108" s="3">
+        <v>7035</v>
+      </c>
+      <c r="O108" s="3">
+        <v>7031</v>
+      </c>
+    </row>
+    <row r="109" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A109" s="4" t="s">
         <v>23</v>
       </c>
@@ -3847,19 +4063,32 @@
       <c r="D109" s="4">
         <v>1</v>
       </c>
-      <c r="E109" s="5"/>
-      <c r="F109" s="4"/>
-      <c r="G109" s="4"/>
+      <c r="E109" s="5">
+        <v>11963</v>
+      </c>
+      <c r="F109" s="4" t="s">
+        <v>120</v>
+      </c>
       <c r="H109" s="4"/>
       <c r="I109" s="4"/>
       <c r="J109" s="4"/>
-      <c r="K109" s="5"/>
-      <c r="L109" s="5"/>
-      <c r="M109" s="4"/>
-      <c r="N109" s="4"/>
-      <c r="O109" s="4"/>
-    </row>
-    <row r="110" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K109" s="5">
+        <v>12061</v>
+      </c>
+      <c r="L109" s="5">
+        <v>11561</v>
+      </c>
+      <c r="M109" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="N109" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="O109" s="4" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="110" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A110" s="1"/>
       <c r="B110" s="1"/>
       <c r="C110" s="1"/>
@@ -3876,7 +4105,7 @@
       <c r="N110" s="1"/>
       <c r="O110" s="1"/>
     </row>
-    <row r="111" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A111" s="1" t="s">
         <v>1</v>
       </c>
@@ -3919,7 +4148,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="112" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A112" s="2" t="s">
         <v>24</v>
       </c>
@@ -3932,19 +4161,33 @@
       <c r="D112" s="2">
         <v>1</v>
       </c>
-      <c r="E112" s="3"/>
-      <c r="F112" s="3"/>
+      <c r="E112" s="3">
+        <v>45542</v>
+      </c>
+      <c r="F112" s="3">
+        <v>7204</v>
+      </c>
       <c r="G112" s="2"/>
       <c r="H112" s="2"/>
       <c r="I112" s="2"/>
       <c r="J112" s="2"/>
-      <c r="K112" s="3"/>
-      <c r="L112" s="3"/>
-      <c r="M112" s="3"/>
-      <c r="N112" s="3"/>
-      <c r="O112" s="3"/>
-    </row>
-    <row r="113" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K112" s="3">
+        <v>49710</v>
+      </c>
+      <c r="L112" s="3">
+        <v>44152</v>
+      </c>
+      <c r="M112" s="3">
+        <v>1821</v>
+      </c>
+      <c r="N112" s="3">
+        <v>7207</v>
+      </c>
+      <c r="O112" s="3">
+        <v>7203</v>
+      </c>
+    </row>
+    <row r="113" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A113" s="4" t="s">
         <v>24</v>
       </c>
@@ -3957,19 +4200,33 @@
       <c r="D113" s="4">
         <v>1</v>
       </c>
-      <c r="E113" s="5"/>
-      <c r="F113" s="4"/>
+      <c r="E113" s="5">
+        <v>11962</v>
+      </c>
+      <c r="F113" s="5">
+        <v>1007</v>
+      </c>
       <c r="G113" s="4"/>
       <c r="H113" s="4"/>
       <c r="I113" s="4"/>
       <c r="J113" s="4"/>
-      <c r="K113" s="5"/>
-      <c r="L113" s="5"/>
-      <c r="M113" s="4"/>
-      <c r="N113" s="5"/>
-      <c r="O113" s="4"/>
-    </row>
-    <row r="114" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K113" s="5">
+        <v>12032</v>
+      </c>
+      <c r="L113" s="5">
+        <v>11564</v>
+      </c>
+      <c r="M113" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="N113" s="5">
+        <v>1012</v>
+      </c>
+      <c r="O113" s="5">
+        <v>1004</v>
+      </c>
+    </row>
+    <row r="114" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A114" s="2" t="s">
         <v>24</v>
       </c>
@@ -3982,19 +4239,33 @@
       <c r="D114" s="2">
         <v>1</v>
       </c>
-      <c r="E114" s="3"/>
-      <c r="F114" s="3"/>
+      <c r="E114" s="3">
+        <v>89125</v>
+      </c>
+      <c r="F114" s="3">
+        <v>7129</v>
+      </c>
       <c r="G114" s="2"/>
       <c r="H114" s="2"/>
       <c r="I114" s="2"/>
       <c r="J114" s="2"/>
-      <c r="K114" s="3"/>
-      <c r="L114" s="3"/>
-      <c r="M114" s="3"/>
-      <c r="N114" s="3"/>
-      <c r="O114" s="3"/>
-    </row>
-    <row r="115" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K114" s="3">
+        <v>94632</v>
+      </c>
+      <c r="L114" s="3">
+        <v>86516</v>
+      </c>
+      <c r="M114" s="3">
+        <v>2652</v>
+      </c>
+      <c r="N114" s="3">
+        <v>7133</v>
+      </c>
+      <c r="O114" s="3">
+        <v>7125</v>
+      </c>
+    </row>
+    <row r="115" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A115" s="4" t="s">
         <v>24</v>
       </c>
@@ -4007,19 +4278,33 @@
       <c r="D115" s="4">
         <v>1</v>
       </c>
-      <c r="E115" s="5"/>
-      <c r="F115" s="4"/>
+      <c r="E115" s="5">
+        <v>11835</v>
+      </c>
+      <c r="F115" s="7">
+        <v>1006</v>
+      </c>
       <c r="G115" s="4"/>
       <c r="H115" s="4"/>
       <c r="I115" s="4"/>
       <c r="J115" s="4"/>
-      <c r="K115" s="5"/>
-      <c r="L115" s="5"/>
-      <c r="M115" s="4"/>
-      <c r="N115" s="5"/>
-      <c r="O115" s="4"/>
-    </row>
-    <row r="116" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K115" s="5">
+        <v>12057</v>
+      </c>
+      <c r="L115" s="5">
+        <v>11549</v>
+      </c>
+      <c r="M115" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="N115" s="5">
+        <v>1008</v>
+      </c>
+      <c r="O115" s="5">
+        <v>1004</v>
+      </c>
+    </row>
+    <row r="116" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A116" s="1"/>
       <c r="B116" s="1"/>
       <c r="C116" s="1"/>
@@ -4036,7 +4321,7 @@
       <c r="N116" s="1"/>
       <c r="O116" s="1"/>
     </row>
-    <row r="117" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A117" s="1" t="s">
         <v>1</v>
       </c>
@@ -4079,7 +4364,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="118" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A118" s="2" t="s">
         <v>25</v>
       </c>
@@ -4092,19 +4377,33 @@
       <c r="D118" s="2">
         <v>1</v>
       </c>
-      <c r="E118" s="3"/>
-      <c r="F118" s="3"/>
+      <c r="E118" s="3">
+        <v>32775</v>
+      </c>
+      <c r="F118" s="3">
+        <v>7380</v>
+      </c>
       <c r="G118" s="2"/>
       <c r="H118" s="2"/>
       <c r="I118" s="2"/>
       <c r="J118" s="2"/>
-      <c r="K118" s="3"/>
-      <c r="L118" s="3"/>
-      <c r="M118" s="3"/>
-      <c r="N118" s="3"/>
-      <c r="O118" s="3"/>
-    </row>
-    <row r="119" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K118" s="3">
+        <v>33740</v>
+      </c>
+      <c r="L118" s="3">
+        <v>31931</v>
+      </c>
+      <c r="M118" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="N118" s="3">
+        <v>7383</v>
+      </c>
+      <c r="O118" s="3">
+        <v>7375</v>
+      </c>
+    </row>
+    <row r="119" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A119" s="4" t="s">
         <v>25</v>
       </c>
@@ -4117,19 +4416,33 @@
       <c r="D119" s="4">
         <v>1</v>
       </c>
-      <c r="E119" s="5"/>
-      <c r="F119" s="4"/>
+      <c r="E119" s="5">
+        <v>11832</v>
+      </c>
+      <c r="F119" s="4" t="s">
+        <v>114</v>
+      </c>
       <c r="G119" s="4"/>
       <c r="H119" s="4"/>
       <c r="I119" s="4"/>
       <c r="J119" s="4"/>
-      <c r="K119" s="5"/>
-      <c r="L119" s="5"/>
-      <c r="M119" s="5"/>
-      <c r="N119" s="4"/>
-      <c r="O119" s="4"/>
-    </row>
-    <row r="120" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K119" s="5">
+        <v>12024</v>
+      </c>
+      <c r="L119" s="5">
+        <v>11531</v>
+      </c>
+      <c r="M119" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="N119" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="O119" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="120" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A120" s="2" t="s">
         <v>25</v>
       </c>
@@ -4142,19 +4455,33 @@
       <c r="D120" s="2">
         <v>1</v>
       </c>
-      <c r="E120" s="3"/>
-      <c r="F120" s="3"/>
+      <c r="E120" s="3">
+        <v>37694</v>
+      </c>
+      <c r="F120" s="3">
+        <v>7524</v>
+      </c>
       <c r="G120" s="2"/>
       <c r="H120" s="2"/>
       <c r="I120" s="2"/>
       <c r="J120" s="2"/>
-      <c r="K120" s="3"/>
-      <c r="L120" s="3"/>
-      <c r="M120" s="3"/>
-      <c r="N120" s="3"/>
-      <c r="O120" s="3"/>
-    </row>
-    <row r="121" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K120" s="3">
+        <v>42121</v>
+      </c>
+      <c r="L120" s="3">
+        <v>36356</v>
+      </c>
+      <c r="M120" s="3">
+        <v>1879</v>
+      </c>
+      <c r="N120" s="3">
+        <v>7527</v>
+      </c>
+      <c r="O120" s="3">
+        <v>7520</v>
+      </c>
+    </row>
+    <row r="121" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A121" s="4" t="s">
         <v>25</v>
       </c>
@@ -4167,19 +4494,33 @@
       <c r="D121" s="4">
         <v>1</v>
       </c>
-      <c r="E121" s="5"/>
-      <c r="F121" s="4"/>
+      <c r="E121" s="5">
+        <v>11681</v>
+      </c>
+      <c r="F121" s="4" t="s">
+        <v>125</v>
+      </c>
       <c r="G121" s="4"/>
       <c r="H121" s="4"/>
       <c r="I121" s="4"/>
       <c r="J121" s="4"/>
-      <c r="K121" s="5"/>
-      <c r="L121" s="5"/>
-      <c r="M121" s="4"/>
-      <c r="N121" s="4"/>
-      <c r="O121" s="4"/>
-    </row>
-    <row r="122" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K121" s="5">
+        <v>12031</v>
+      </c>
+      <c r="L121" s="5">
+        <v>11503</v>
+      </c>
+      <c r="M121" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="N121" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="O121" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="122" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A122" s="1"/>
       <c r="B122" s="1"/>
       <c r="C122" s="1"/>
@@ -4196,7 +4537,7 @@
       <c r="N122" s="1"/>
       <c r="O122" s="1"/>
     </row>
-    <row r="123" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A123" s="1" t="s">
         <v>1</v>
       </c>
@@ -4239,7 +4580,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="124" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A124" s="2" t="s">
         <v>26</v>
       </c>
@@ -4252,19 +4593,33 @@
       <c r="D124" s="2">
         <v>1</v>
       </c>
-      <c r="E124" s="3"/>
-      <c r="F124" s="3"/>
+      <c r="E124" s="3">
+        <v>33328</v>
+      </c>
+      <c r="F124" s="3">
+        <v>7207</v>
+      </c>
       <c r="G124" s="2"/>
       <c r="H124" s="2"/>
       <c r="I124" s="2"/>
       <c r="J124" s="2"/>
-      <c r="K124" s="3"/>
-      <c r="L124" s="3"/>
-      <c r="M124" s="3"/>
-      <c r="N124" s="3"/>
-      <c r="O124" s="3"/>
-    </row>
-    <row r="125" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K124" s="3">
+        <v>36354</v>
+      </c>
+      <c r="L124" s="3">
+        <v>32093</v>
+      </c>
+      <c r="M124" s="3">
+        <v>1524</v>
+      </c>
+      <c r="N124" s="3">
+        <v>7211</v>
+      </c>
+      <c r="O124" s="3">
+        <v>7203</v>
+      </c>
+    </row>
+    <row r="125" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A125" s="4" t="s">
         <v>26</v>
       </c>
@@ -4277,19 +4632,33 @@
       <c r="D125" s="4">
         <v>1</v>
       </c>
-      <c r="E125" s="5"/>
-      <c r="F125" s="5"/>
+      <c r="E125" s="5">
+        <v>11956</v>
+      </c>
+      <c r="F125" s="5">
+        <v>1096</v>
+      </c>
       <c r="G125" s="4"/>
       <c r="H125" s="4"/>
       <c r="I125" s="4"/>
       <c r="J125" s="4"/>
-      <c r="K125" s="5"/>
-      <c r="L125" s="5"/>
-      <c r="M125" s="4"/>
-      <c r="N125" s="5"/>
-      <c r="O125" s="5"/>
-    </row>
-    <row r="126" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K125" s="5">
+        <v>12938</v>
+      </c>
+      <c r="L125" s="5">
+        <v>11502</v>
+      </c>
+      <c r="M125" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="N125" s="5">
+        <v>1098</v>
+      </c>
+      <c r="O125" s="5">
+        <v>1094</v>
+      </c>
+    </row>
+    <row r="126" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A126" s="2" t="s">
         <v>26</v>
       </c>
@@ -4302,19 +4671,33 @@
       <c r="D126" s="2">
         <v>1</v>
       </c>
-      <c r="E126" s="3"/>
-      <c r="F126" s="3"/>
+      <c r="E126" s="3">
+        <v>38423</v>
+      </c>
+      <c r="F126" s="3">
+        <v>7594</v>
+      </c>
       <c r="G126" s="2"/>
       <c r="H126" s="2"/>
       <c r="I126" s="2"/>
       <c r="J126" s="2"/>
-      <c r="K126" s="3"/>
-      <c r="L126" s="3"/>
-      <c r="M126" s="3"/>
-      <c r="N126" s="3"/>
-      <c r="O126" s="3"/>
-    </row>
-    <row r="127" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K126" s="3">
+        <v>41291</v>
+      </c>
+      <c r="L126" s="3">
+        <v>35695</v>
+      </c>
+      <c r="M126" s="3">
+        <v>2168</v>
+      </c>
+      <c r="N126" s="3">
+        <v>7594</v>
+      </c>
+      <c r="O126" s="3">
+        <v>7594</v>
+      </c>
+    </row>
+    <row r="127" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A127" s="4" t="s">
         <v>26</v>
       </c>
@@ -4327,24 +4710,38 @@
       <c r="D127" s="4">
         <v>1</v>
       </c>
-      <c r="E127" s="5"/>
-      <c r="F127" s="5"/>
+      <c r="E127" s="5">
+        <v>12029</v>
+      </c>
+      <c r="F127" s="5">
+        <v>1022</v>
+      </c>
       <c r="G127" s="4"/>
       <c r="H127" s="4"/>
       <c r="I127" s="4"/>
       <c r="J127" s="4"/>
-      <c r="K127" s="5"/>
-      <c r="L127" s="5"/>
-      <c r="M127" s="4"/>
-      <c r="N127" s="5"/>
-      <c r="O127" s="5"/>
-    </row>
-    <row r="135" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K127" s="5">
+        <v>12547</v>
+      </c>
+      <c r="L127" s="5">
+        <v>11725</v>
+      </c>
+      <c r="M127" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="N127" s="5">
+        <v>1023</v>
+      </c>
+      <c r="O127" s="5">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="135" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A135">
         <v>2025</v>
       </c>
     </row>
-    <row r="137" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A137" s="1" t="s">
         <v>1</v>
       </c>
@@ -4387,7 +4784,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="138" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A138" s="2" t="s">
         <v>9</v>
       </c>
@@ -4400,19 +4797,33 @@
       <c r="D138" s="2">
         <v>1</v>
       </c>
-      <c r="E138" s="3"/>
-      <c r="F138" s="3"/>
+      <c r="E138" s="3">
+        <v>33673</v>
+      </c>
+      <c r="F138" s="3">
+        <v>6918</v>
+      </c>
       <c r="G138" s="2"/>
       <c r="H138" s="2"/>
       <c r="I138" s="2"/>
       <c r="J138" s="2"/>
-      <c r="K138" s="3"/>
-      <c r="L138" s="3"/>
-      <c r="M138" s="3"/>
-      <c r="N138" s="3"/>
-      <c r="O138" s="3"/>
-    </row>
-    <row r="139" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K138" s="3">
+        <v>36874</v>
+      </c>
+      <c r="L138" s="3">
+        <v>32358</v>
+      </c>
+      <c r="M138" s="3">
+        <v>1560</v>
+      </c>
+      <c r="N138" s="3">
+        <v>6922</v>
+      </c>
+      <c r="O138" s="3">
+        <v>6914</v>
+      </c>
+    </row>
+    <row r="139" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A139" s="4" t="s">
         <v>9</v>
       </c>
@@ -4425,19 +4836,33 @@
       <c r="D139" s="4">
         <v>1</v>
       </c>
-      <c r="E139" s="5"/>
-      <c r="F139" s="4"/>
+      <c r="E139" s="5">
+        <v>12002</v>
+      </c>
+      <c r="F139" s="4" t="s">
+        <v>109</v>
+      </c>
       <c r="G139" s="4"/>
       <c r="H139" s="4"/>
       <c r="I139" s="4"/>
       <c r="J139" s="4"/>
-      <c r="K139" s="5"/>
-      <c r="L139" s="5"/>
-      <c r="M139" s="4"/>
-      <c r="N139" s="4"/>
-      <c r="O139" s="4"/>
-    </row>
-    <row r="140" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K139" s="5">
+        <v>12041</v>
+      </c>
+      <c r="L139" s="5">
+        <v>11960</v>
+      </c>
+      <c r="M139" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="N139" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="O139" s="4" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="140" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A140" s="2" t="s">
         <v>9</v>
       </c>
@@ -4450,19 +4875,33 @@
       <c r="D140" s="2">
         <v>1</v>
       </c>
-      <c r="E140" s="3"/>
-      <c r="F140" s="3"/>
+      <c r="E140" s="3">
+        <v>33666</v>
+      </c>
+      <c r="F140" s="3">
+        <v>7141</v>
+      </c>
       <c r="G140" s="2"/>
       <c r="H140" s="2"/>
       <c r="I140" s="2"/>
       <c r="J140" s="2"/>
-      <c r="K140" s="3"/>
-      <c r="L140" s="3"/>
-      <c r="M140" s="3"/>
-      <c r="N140" s="3"/>
-      <c r="O140" s="3"/>
-    </row>
-    <row r="141" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K140" s="3">
+        <v>35946</v>
+      </c>
+      <c r="L140" s="3">
+        <v>33092</v>
+      </c>
+      <c r="M140" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="N140" s="3">
+        <v>7145</v>
+      </c>
+      <c r="O140" s="3">
+        <v>7137</v>
+      </c>
+    </row>
+    <row r="141" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A141" s="4" t="s">
         <v>9</v>
       </c>
@@ -4475,19 +4914,33 @@
       <c r="D141" s="4">
         <v>1</v>
       </c>
-      <c r="E141" s="5"/>
-      <c r="F141" s="4"/>
+      <c r="E141" s="5">
+        <v>11990</v>
+      </c>
+      <c r="F141" s="4" t="s">
+        <v>136</v>
+      </c>
       <c r="G141" s="4"/>
       <c r="H141" s="4"/>
       <c r="I141" s="4"/>
       <c r="J141" s="4"/>
-      <c r="K141" s="5"/>
-      <c r="L141" s="5"/>
-      <c r="M141" s="4"/>
-      <c r="N141" s="4"/>
-      <c r="O141" s="4"/>
-    </row>
-    <row r="142" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K141" s="5">
+        <v>12579</v>
+      </c>
+      <c r="L141" s="5">
+        <v>11493</v>
+      </c>
+      <c r="M141" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="N141" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="O141" s="4" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="142" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A142" s="1"/>
       <c r="B142" s="1"/>
       <c r="C142" s="1"/>
@@ -4504,7 +4957,7 @@
       <c r="N142" s="1"/>
       <c r="O142" s="1"/>
     </row>
-    <row r="143" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A143" s="1" t="s">
         <v>1</v>
       </c>
@@ -4547,7 +5000,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="144" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A144" s="2" t="s">
         <v>23</v>
       </c>
@@ -4560,19 +5013,33 @@
       <c r="D144" s="2">
         <v>1</v>
       </c>
-      <c r="E144" s="3"/>
-      <c r="F144" s="3"/>
+      <c r="E144" s="3">
+        <v>100091</v>
+      </c>
+      <c r="F144" s="3">
+        <v>15828</v>
+      </c>
       <c r="G144" s="2"/>
       <c r="H144" s="2"/>
       <c r="I144" s="2"/>
       <c r="J144" s="2"/>
-      <c r="K144" s="3"/>
-      <c r="L144" s="3"/>
-      <c r="M144" s="3"/>
-      <c r="N144" s="3"/>
-      <c r="O144" s="3"/>
-    </row>
-    <row r="145" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K144" s="3">
+        <v>106628</v>
+      </c>
+      <c r="L144" s="3">
+        <v>95986</v>
+      </c>
+      <c r="M144" s="3">
+        <v>3924</v>
+      </c>
+      <c r="N144" s="3">
+        <v>15832</v>
+      </c>
+      <c r="O144" s="3">
+        <v>15824</v>
+      </c>
+    </row>
+    <row r="145" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A145" s="4" t="s">
         <v>23</v>
       </c>
@@ -4585,19 +5052,33 @@
       <c r="D145" s="4">
         <v>1</v>
       </c>
-      <c r="E145" s="5"/>
-      <c r="F145" s="5"/>
+      <c r="E145" s="5">
+        <v>22595</v>
+      </c>
+      <c r="F145" s="5">
+        <v>2006</v>
+      </c>
       <c r="G145" s="4"/>
       <c r="H145" s="4"/>
       <c r="I145" s="4"/>
       <c r="J145" s="4"/>
-      <c r="K145" s="5"/>
-      <c r="L145" s="5"/>
-      <c r="M145" s="4"/>
-      <c r="N145" s="5"/>
-      <c r="O145" s="5"/>
-    </row>
-    <row r="146" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K145" s="5">
+        <v>23428</v>
+      </c>
+      <c r="L145" s="5">
+        <v>22036</v>
+      </c>
+      <c r="M145" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="N145" s="5">
+        <v>2008</v>
+      </c>
+      <c r="O145" s="5">
+        <v>2004</v>
+      </c>
+    </row>
+    <row r="146" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A146" s="2" t="s">
         <v>23</v>
       </c>
@@ -4610,19 +5091,33 @@
       <c r="D146" s="2">
         <v>1</v>
       </c>
-      <c r="E146" s="3"/>
-      <c r="F146" s="3"/>
+      <c r="E146" s="3">
+        <v>147632</v>
+      </c>
+      <c r="F146" s="3">
+        <v>15464</v>
+      </c>
       <c r="G146" s="2"/>
       <c r="H146" s="2"/>
       <c r="I146" s="2"/>
       <c r="J146" s="2"/>
-      <c r="K146" s="3"/>
-      <c r="L146" s="3"/>
-      <c r="M146" s="3"/>
-      <c r="N146" s="3"/>
-      <c r="O146" s="3"/>
-    </row>
-    <row r="147" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K146" s="3">
+        <v>154267</v>
+      </c>
+      <c r="L146" s="3">
+        <v>141017</v>
+      </c>
+      <c r="M146" s="3">
+        <v>4158</v>
+      </c>
+      <c r="N146" s="3">
+        <v>15469</v>
+      </c>
+      <c r="O146" s="3">
+        <v>15457</v>
+      </c>
+    </row>
+    <row r="147" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A147" s="4" t="s">
         <v>23</v>
       </c>
@@ -4635,19 +5130,33 @@
       <c r="D147" s="4">
         <v>1</v>
       </c>
-      <c r="E147" s="5"/>
-      <c r="F147" s="4"/>
+      <c r="E147" s="5">
+        <v>13003</v>
+      </c>
+      <c r="F147" s="4" t="s">
+        <v>138</v>
+      </c>
       <c r="G147" s="4"/>
       <c r="H147" s="4"/>
       <c r="I147" s="4"/>
       <c r="J147" s="4"/>
-      <c r="K147" s="5"/>
-      <c r="L147" s="5"/>
-      <c r="M147" s="5"/>
-      <c r="N147" s="4"/>
-      <c r="O147" s="4"/>
-    </row>
-    <row r="148" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K147" s="5">
+        <v>22030</v>
+      </c>
+      <c r="L147" s="5">
+        <v>11971</v>
+      </c>
+      <c r="M147" s="5">
+        <v>3172</v>
+      </c>
+      <c r="N147" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="O147" s="4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="148" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A148" s="1"/>
       <c r="B148" s="1"/>
       <c r="C148" s="1"/>
@@ -4664,7 +5173,7 @@
       <c r="N148" s="1"/>
       <c r="O148" s="1"/>
     </row>
-    <row r="149" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A149" s="1" t="s">
         <v>1</v>
       </c>
@@ -4707,7 +5216,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="150" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A150" s="2" t="s">
         <v>53</v>
       </c>
@@ -4720,19 +5229,33 @@
       <c r="D150" s="2">
         <v>1</v>
       </c>
-      <c r="E150" s="3"/>
-      <c r="F150" s="3"/>
+      <c r="E150" s="3">
+        <v>34758</v>
+      </c>
+      <c r="F150" s="3">
+        <v>7095</v>
+      </c>
       <c r="G150" s="2"/>
       <c r="H150" s="2"/>
       <c r="I150" s="2"/>
       <c r="J150" s="2"/>
-      <c r="K150" s="3"/>
-      <c r="L150" s="3"/>
-      <c r="M150" s="2"/>
-      <c r="N150" s="3"/>
-      <c r="O150" s="3"/>
-    </row>
-    <row r="151" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K150" s="3">
+        <v>36002</v>
+      </c>
+      <c r="L150" s="3">
+        <v>34131</v>
+      </c>
+      <c r="M150" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="N150" s="3">
+        <v>7098</v>
+      </c>
+      <c r="O150" s="3">
+        <v>7094</v>
+      </c>
+    </row>
+    <row r="151" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A151" s="4" t="s">
         <v>53</v>
       </c>
@@ -4745,19 +5268,33 @@
       <c r="D151" s="4">
         <v>1</v>
       </c>
-      <c r="E151" s="5"/>
-      <c r="F151" s="4"/>
+      <c r="E151" s="5">
+        <v>11999</v>
+      </c>
+      <c r="F151" s="4" t="s">
+        <v>45</v>
+      </c>
       <c r="G151" s="4"/>
       <c r="H151" s="4"/>
       <c r="I151" s="4"/>
       <c r="J151" s="4"/>
-      <c r="K151" s="5"/>
-      <c r="L151" s="5"/>
-      <c r="M151" s="4"/>
-      <c r="N151" s="4"/>
-      <c r="O151" s="4"/>
-    </row>
-    <row r="152" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K151" s="5">
+        <v>12064</v>
+      </c>
+      <c r="L151" s="5">
+        <v>11941</v>
+      </c>
+      <c r="M151" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="N151" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="O151" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="152" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A152" s="2" t="s">
         <v>53</v>
       </c>
@@ -4770,19 +5307,33 @@
       <c r="D152" s="2">
         <v>1</v>
       </c>
-      <c r="E152" s="3"/>
-      <c r="F152" s="3"/>
+      <c r="E152" s="3">
+        <v>37838</v>
+      </c>
+      <c r="F152" s="3">
+        <v>7157</v>
+      </c>
       <c r="G152" s="2"/>
       <c r="H152" s="2"/>
       <c r="I152" s="2"/>
       <c r="J152" s="2"/>
-      <c r="K152" s="3"/>
-      <c r="L152" s="3"/>
-      <c r="M152" s="3"/>
-      <c r="N152" s="3"/>
-      <c r="O152" s="3"/>
-    </row>
-    <row r="153" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K152" s="3">
+        <v>42000</v>
+      </c>
+      <c r="L152" s="3">
+        <v>36281</v>
+      </c>
+      <c r="M152" s="3">
+        <v>1761</v>
+      </c>
+      <c r="N152" s="3">
+        <v>7160</v>
+      </c>
+      <c r="O152" s="3">
+        <v>7156</v>
+      </c>
+    </row>
+    <row r="153" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A153" s="4" t="s">
         <v>53</v>
       </c>
@@ -4796,10 +5347,10 @@
         <v>1</v>
       </c>
       <c r="E153" s="5">
-        <v>12101</v>
+        <v>13271</v>
       </c>
       <c r="F153" s="5">
-        <v>1031</v>
+        <v>1018</v>
       </c>
       <c r="G153" s="4">
         <v>96</v>
@@ -4810,22 +5361,22 @@
       <c r="I153" s="4"/>
       <c r="J153" s="4"/>
       <c r="K153" s="5">
-        <v>12833</v>
+        <v>24009</v>
       </c>
       <c r="L153" s="5">
-        <v>11989</v>
-      </c>
-      <c r="M153" s="4" t="s">
-        <v>73</v>
+        <v>11975</v>
+      </c>
+      <c r="M153" s="5">
+        <v>3775</v>
       </c>
       <c r="N153" s="5">
-        <v>1039</v>
+        <v>1020</v>
       </c>
       <c r="O153" s="5">
-        <v>1027</v>
-      </c>
-    </row>
-    <row r="154" spans="1:15" x14ac:dyDescent="0.25">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="154" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A154" s="1"/>
       <c r="B154" s="1"/>
       <c r="C154" s="1"/>
@@ -4842,7 +5393,7 @@
       <c r="N154" s="1"/>
       <c r="O154" s="1"/>
     </row>
-    <row r="155" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A155" s="1" t="s">
         <v>1</v>
       </c>
@@ -4885,7 +5436,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="156" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A156" s="2" t="s">
         <v>54</v>
       </c>
@@ -4898,19 +5449,33 @@
       <c r="D156" s="2">
         <v>1</v>
       </c>
-      <c r="E156" s="3"/>
-      <c r="F156" s="3"/>
+      <c r="E156" s="3">
+        <v>32560</v>
+      </c>
+      <c r="F156" s="3">
+        <v>6953</v>
+      </c>
       <c r="G156" s="2"/>
       <c r="H156" s="2"/>
       <c r="I156" s="2"/>
       <c r="J156" s="2"/>
-      <c r="K156" s="3"/>
-      <c r="L156" s="3"/>
-      <c r="M156" s="3"/>
-      <c r="N156" s="3"/>
-      <c r="O156" s="3"/>
-    </row>
-    <row r="157" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K156" s="3">
+        <v>34333</v>
+      </c>
+      <c r="L156" s="3">
+        <v>30833</v>
+      </c>
+      <c r="M156" s="3">
+        <v>1068</v>
+      </c>
+      <c r="N156" s="3">
+        <v>6953</v>
+      </c>
+      <c r="O156" s="3">
+        <v>6949</v>
+      </c>
+    </row>
+    <row r="157" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A157" s="4" t="s">
         <v>54</v>
       </c>
@@ -4923,19 +5488,33 @@
       <c r="D157" s="4">
         <v>1</v>
       </c>
-      <c r="E157" s="5"/>
-      <c r="F157" s="4"/>
+      <c r="E157" s="5">
+        <v>12365</v>
+      </c>
+      <c r="F157" s="4" t="s">
+        <v>61</v>
+      </c>
       <c r="G157" s="4"/>
       <c r="H157" s="4"/>
       <c r="I157" s="4"/>
       <c r="J157" s="4"/>
-      <c r="K157" s="5"/>
-      <c r="L157" s="5"/>
-      <c r="M157" s="4"/>
-      <c r="N157" s="4"/>
-      <c r="O157" s="4"/>
-    </row>
-    <row r="158" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K157" s="5">
+        <v>13840</v>
+      </c>
+      <c r="L157" s="5">
+        <v>11954</v>
+      </c>
+      <c r="M157" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="N157" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="O157" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="158" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A158" s="2" t="s">
         <v>54</v>
       </c>
@@ -4948,19 +5527,33 @@
       <c r="D158" s="2">
         <v>1</v>
       </c>
-      <c r="E158" s="3"/>
-      <c r="F158" s="3"/>
+      <c r="E158" s="3">
+        <v>36393</v>
+      </c>
+      <c r="F158" s="3">
+        <v>7878</v>
+      </c>
       <c r="G158" s="2"/>
       <c r="H158" s="2"/>
       <c r="I158" s="2"/>
       <c r="J158" s="2"/>
-      <c r="K158" s="3"/>
-      <c r="L158" s="3"/>
-      <c r="M158" s="3"/>
-      <c r="N158" s="3"/>
-      <c r="O158" s="3"/>
-    </row>
-    <row r="159" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K158" s="3">
+        <v>40551</v>
+      </c>
+      <c r="L158" s="3">
+        <v>35461</v>
+      </c>
+      <c r="M158" s="3">
+        <v>1515</v>
+      </c>
+      <c r="N158" s="3">
+        <v>7883</v>
+      </c>
+      <c r="O158" s="3">
+        <v>7875</v>
+      </c>
+    </row>
+    <row r="159" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A159" s="4" t="s">
         <v>54</v>
       </c>
@@ -4973,19 +5566,33 @@
       <c r="D159" s="4">
         <v>1</v>
       </c>
-      <c r="E159" s="5"/>
-      <c r="F159" s="5"/>
+      <c r="E159" s="5">
+        <v>11997</v>
+      </c>
+      <c r="F159" s="5">
+        <v>1026</v>
+      </c>
       <c r="G159" s="4"/>
       <c r="H159" s="4"/>
       <c r="I159" s="4"/>
       <c r="J159" s="4"/>
-      <c r="K159" s="5"/>
-      <c r="L159" s="5"/>
-      <c r="M159" s="4"/>
-      <c r="N159" s="5"/>
-      <c r="O159" s="5"/>
-    </row>
-    <row r="160" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K159" s="5">
+        <v>12107</v>
+      </c>
+      <c r="L159" s="5">
+        <v>11923</v>
+      </c>
+      <c r="M159" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="N159" s="5">
+        <v>1027</v>
+      </c>
+      <c r="O159" s="5">
+        <v>1023</v>
+      </c>
+    </row>
+    <row r="160" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A160" s="1"/>
       <c r="B160" s="1"/>
       <c r="C160" s="1"/>
@@ -5002,7 +5609,7 @@
       <c r="N160" s="1"/>
       <c r="O160" s="1"/>
     </row>
-    <row r="161" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A161" s="1" t="s">
         <v>1</v>
       </c>
@@ -5045,7 +5652,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="162" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A162" s="2" t="s">
         <v>55</v>
       </c>
@@ -5058,19 +5665,33 @@
       <c r="D162" s="2">
         <v>1</v>
       </c>
-      <c r="E162" s="3"/>
-      <c r="F162" s="3"/>
+      <c r="E162" s="3">
+        <v>34288</v>
+      </c>
+      <c r="F162" s="3">
+        <v>7207</v>
+      </c>
       <c r="G162" s="2"/>
       <c r="H162" s="2"/>
       <c r="I162" s="2"/>
       <c r="J162" s="2"/>
-      <c r="K162" s="3"/>
-      <c r="L162" s="3"/>
-      <c r="M162" s="3"/>
-      <c r="N162" s="3"/>
-      <c r="O162" s="3"/>
-    </row>
-    <row r="163" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K162" s="3">
+        <v>40336</v>
+      </c>
+      <c r="L162" s="3">
+        <v>32366</v>
+      </c>
+      <c r="M162" s="3">
+        <v>2593</v>
+      </c>
+      <c r="N162" s="3">
+        <v>7215</v>
+      </c>
+      <c r="O162" s="3">
+        <v>7203</v>
+      </c>
+    </row>
+    <row r="163" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A163" s="4" t="s">
         <v>55</v>
       </c>
@@ -5083,19 +5704,33 @@
       <c r="D163" s="4">
         <v>1</v>
       </c>
-      <c r="E163" s="5"/>
-      <c r="F163" s="5"/>
+      <c r="E163" s="5">
+        <v>12001</v>
+      </c>
+      <c r="F163" s="5">
+        <v>1278</v>
+      </c>
       <c r="G163" s="4"/>
       <c r="H163" s="4"/>
       <c r="I163" s="4"/>
       <c r="J163" s="4"/>
-      <c r="K163" s="5"/>
-      <c r="L163" s="5"/>
-      <c r="M163" s="5"/>
-      <c r="N163" s="5"/>
-      <c r="O163" s="5"/>
-    </row>
-    <row r="164" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K163" s="5">
+        <v>12037</v>
+      </c>
+      <c r="L163" s="5">
+        <v>11966</v>
+      </c>
+      <c r="M163" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="N163" s="5">
+        <v>1281</v>
+      </c>
+      <c r="O163" s="5">
+        <v>1273</v>
+      </c>
+    </row>
+    <row r="164" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A164" s="2" t="s">
         <v>55</v>
       </c>
@@ -5108,19 +5743,33 @@
       <c r="D164" s="2">
         <v>1</v>
       </c>
-      <c r="E164" s="3"/>
-      <c r="F164" s="3"/>
+      <c r="E164" s="3">
+        <v>32506</v>
+      </c>
+      <c r="F164" s="3">
+        <v>7207</v>
+      </c>
       <c r="G164" s="2"/>
       <c r="H164" s="2"/>
       <c r="I164" s="2"/>
       <c r="J164" s="2"/>
-      <c r="K164" s="3"/>
-      <c r="L164" s="3"/>
-      <c r="M164" s="3"/>
-      <c r="N164" s="3"/>
-      <c r="O164" s="3"/>
-    </row>
-    <row r="165" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K164" s="3">
+        <v>33355</v>
+      </c>
+      <c r="L164" s="3">
+        <v>32135</v>
+      </c>
+      <c r="M164" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="N164" s="3">
+        <v>7211</v>
+      </c>
+      <c r="O164" s="3">
+        <v>7203</v>
+      </c>
+    </row>
+    <row r="165" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A165" s="4" t="s">
         <v>55</v>
       </c>
@@ -5133,19 +5782,33 @@
       <c r="D165" s="4">
         <v>1</v>
       </c>
-      <c r="E165" s="5"/>
-      <c r="F165" s="5"/>
+      <c r="E165" s="5">
+        <v>11911</v>
+      </c>
+      <c r="F165" s="5">
+        <v>1273</v>
+      </c>
       <c r="G165" s="4"/>
       <c r="H165" s="4"/>
       <c r="I165" s="4"/>
       <c r="J165" s="4"/>
-      <c r="K165" s="5"/>
-      <c r="L165" s="5"/>
-      <c r="M165" s="4"/>
-      <c r="N165" s="5"/>
-      <c r="O165" s="5"/>
-    </row>
-    <row r="166" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K165" s="5">
+        <v>12049</v>
+      </c>
+      <c r="L165" s="5">
+        <v>11524</v>
+      </c>
+      <c r="M165" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="N165" s="5">
+        <v>1273</v>
+      </c>
+      <c r="O165" s="5">
+        <v>1270</v>
+      </c>
+    </row>
+    <row r="166" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A166" s="1"/>
       <c r="B166" s="1"/>
       <c r="C166" s="1"/>
@@ -5162,12 +5825,12 @@
       <c r="N166" s="1"/>
       <c r="O166" s="1"/>
     </row>
-    <row r="183" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="184" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A184">
         <v>2024</v>
       </c>

</xml_diff>

<commit_message>
added algorithms to results
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/21c1a4ced64a9754/Documents/Uni/Bachelor Thesis/BachelorThesis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="287" documentId="13_ncr:1_{30350997-3BBF-49AB-916C-212AA2CBCFFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A8736EF-0517-47FB-A85B-0A84D8E72BDF}"/>
+  <xr:revisionPtr revIDLastSave="341" documentId="13_ncr:1_{30350997-3BBF-49AB-916C-212AA2CBCFFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{86315208-3E9E-4B82-8859-205CA8B4FD4B}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{2A4234DB-3A22-4351-83C3-53CA1AE1142A}"/>
+    <workbookView xWindow="12390" yWindow="0" windowWidth="12660" windowHeight="16010" xr2:uid="{2A4234DB-3A22-4351-83C3-53CA1AE1142A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="734" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="773" uniqueCount="161">
   <si>
     <t>Benchmarking results LLMs</t>
   </si>
@@ -459,6 +459,66 @@
   </si>
   <si>
     <t xml:space="preserve"> 0.191 </t>
+  </si>
+  <si>
+    <t>Hashmap based frequency counting</t>
+  </si>
+  <si>
+    <t>Brute force with sliding window difference check</t>
+  </si>
+  <si>
+    <t>BFS flood fill algorithm</t>
+  </si>
+  <si>
+    <t>cramers rule</t>
+  </si>
+  <si>
+    <t>rule based validation/constraint checking on a graph</t>
+  </si>
+  <si>
+    <t>Brute force with monotonicity check</t>
+  </si>
+  <si>
+    <t>DFS flood fill algorithm</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> cramers rule + extended euclidian algorithm</t>
+  </si>
+  <si>
+    <t>graph based pattern matching</t>
+  </si>
+  <si>
+    <t>cramers rule + extended euclidean algorithm</t>
+  </si>
+  <si>
+    <t>graph based circuit reconstruction</t>
+  </si>
+  <si>
+    <t>Simulation with modular arithmetic</t>
+  </si>
+  <si>
+    <t>Precomputation + prefix sums with binary search</t>
+  </si>
+  <si>
+    <t>grid parsing with column wise aggregation</t>
+  </si>
+  <si>
+    <t>dynamic programming</t>
+  </si>
+  <si>
+    <t>dynamic programming with memoization</t>
+  </si>
+  <si>
+    <t>precomputaion + two pointer technique</t>
+  </si>
+  <si>
+    <t>grid parsing with column wise scan</t>
+  </si>
+  <si>
+    <t>precomuputation with brute force range query</t>
+  </si>
+  <si>
+    <t>precomputation with brute force filtering</t>
   </si>
 </sst>
 </file>
@@ -468,7 +528,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000E+00"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -486,6 +546,14 @@
     <font>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -523,7 +591,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -544,6 +612,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Bad" xfId="2" builtinId="27"/>
@@ -561,6 +632,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3737,7 +3812,9 @@
         <v>6984</v>
       </c>
       <c r="G100" s="2"/>
-      <c r="H100" s="2"/>
+      <c r="H100" s="2" t="s">
+        <v>141</v>
+      </c>
       <c r="I100" s="2"/>
       <c r="J100" s="2"/>
       <c r="K100" s="3">
@@ -3776,7 +3853,9 @@
         <v>106</v>
       </c>
       <c r="G101" s="4"/>
-      <c r="H101" s="4"/>
+      <c r="H101" s="4" t="s">
+        <v>141</v>
+      </c>
       <c r="I101" s="4"/>
       <c r="J101" s="4"/>
       <c r="K101" s="5">
@@ -3815,7 +3894,9 @@
         <v>7305</v>
       </c>
       <c r="G102" s="2"/>
-      <c r="H102" s="2"/>
+      <c r="H102" s="2" t="s">
+        <v>141</v>
+      </c>
       <c r="I102" s="2"/>
       <c r="J102" s="2"/>
       <c r="K102" s="3">
@@ -3854,7 +3935,9 @@
         <v>114</v>
       </c>
       <c r="G103" s="4"/>
-      <c r="H103" s="4"/>
+      <c r="H103" s="4" t="s">
+        <v>141</v>
+      </c>
       <c r="I103" s="4"/>
       <c r="J103" s="4"/>
       <c r="K103" s="5">
@@ -3953,7 +4036,9 @@
         <v>6973</v>
       </c>
       <c r="G106" s="2"/>
-      <c r="H106" s="2"/>
+      <c r="H106" s="2" t="s">
+        <v>146</v>
+      </c>
       <c r="I106" s="2"/>
       <c r="J106" s="2"/>
       <c r="K106" s="3">
@@ -3992,7 +4077,9 @@
         <v>109</v>
       </c>
       <c r="G107" s="4"/>
-      <c r="H107" s="4"/>
+      <c r="H107" s="4" t="s">
+        <v>146</v>
+      </c>
       <c r="I107" s="4"/>
       <c r="J107" s="4"/>
       <c r="K107" s="5">
@@ -4031,7 +4118,9 @@
         <v>7034</v>
       </c>
       <c r="G108" s="2"/>
-      <c r="H108" s="2"/>
+      <c r="H108" s="2" t="s">
+        <v>142</v>
+      </c>
       <c r="I108" s="2"/>
       <c r="J108" s="2"/>
       <c r="K108" s="3">
@@ -4069,7 +4158,9 @@
       <c r="F109" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="H109" s="4"/>
+      <c r="H109" s="4" t="s">
+        <v>142</v>
+      </c>
       <c r="I109" s="4"/>
       <c r="J109" s="4"/>
       <c r="K109" s="5">
@@ -4168,7 +4259,9 @@
         <v>7204</v>
       </c>
       <c r="G112" s="2"/>
-      <c r="H112" s="2"/>
+      <c r="H112" t="s">
+        <v>147</v>
+      </c>
       <c r="I112" s="2"/>
       <c r="J112" s="2"/>
       <c r="K112" s="3">
@@ -4207,7 +4300,9 @@
         <v>1007</v>
       </c>
       <c r="G113" s="4"/>
-      <c r="H113" s="4"/>
+      <c r="H113" s="4" t="s">
+        <v>143</v>
+      </c>
       <c r="I113" s="4"/>
       <c r="J113" s="4"/>
       <c r="K113" s="5">
@@ -4246,7 +4341,9 @@
         <v>7129</v>
       </c>
       <c r="G114" s="2"/>
-      <c r="H114" s="2"/>
+      <c r="H114" s="2" t="s">
+        <v>143</v>
+      </c>
       <c r="I114" s="2"/>
       <c r="J114" s="2"/>
       <c r="K114" s="3">
@@ -4285,7 +4382,9 @@
         <v>1006</v>
       </c>
       <c r="G115" s="4"/>
-      <c r="H115" s="4"/>
+      <c r="H115" s="4" t="s">
+        <v>143</v>
+      </c>
       <c r="I115" s="4"/>
       <c r="J115" s="4"/>
       <c r="K115" s="5">
@@ -4384,7 +4483,9 @@
         <v>7380</v>
       </c>
       <c r="G118" s="2"/>
-      <c r="H118" s="2"/>
+      <c r="H118" s="2" t="s">
+        <v>148</v>
+      </c>
       <c r="I118" s="2"/>
       <c r="J118" s="2"/>
       <c r="K118" s="3">
@@ -4423,7 +4524,9 @@
         <v>114</v>
       </c>
       <c r="G119" s="4"/>
-      <c r="H119" s="4"/>
+      <c r="H119" s="4" t="s">
+        <v>150</v>
+      </c>
       <c r="I119" s="4"/>
       <c r="J119" s="4"/>
       <c r="K119" s="5">
@@ -4462,7 +4565,9 @@
         <v>7524</v>
       </c>
       <c r="G120" s="2"/>
-      <c r="H120" s="2"/>
+      <c r="H120" s="2" t="s">
+        <v>144</v>
+      </c>
       <c r="I120" s="2"/>
       <c r="J120" s="2"/>
       <c r="K120" s="3">
@@ -4501,7 +4606,9 @@
         <v>125</v>
       </c>
       <c r="G121" s="4"/>
-      <c r="H121" s="4"/>
+      <c r="H121" s="4" t="s">
+        <v>144</v>
+      </c>
       <c r="I121" s="4"/>
       <c r="J121" s="4"/>
       <c r="K121" s="5">
@@ -4600,7 +4707,9 @@
         <v>7207</v>
       </c>
       <c r="G124" s="2"/>
-      <c r="H124" s="2"/>
+      <c r="H124" s="2" t="s">
+        <v>149</v>
+      </c>
       <c r="I124" s="2"/>
       <c r="J124" s="2"/>
       <c r="K124" s="3">
@@ -4639,7 +4748,9 @@
         <v>1096</v>
       </c>
       <c r="G125" s="4"/>
-      <c r="H125" s="4"/>
+      <c r="H125" s="4" t="s">
+        <v>151</v>
+      </c>
       <c r="I125" s="4"/>
       <c r="J125" s="4"/>
       <c r="K125" s="5">
@@ -4678,7 +4789,9 @@
         <v>7594</v>
       </c>
       <c r="G126" s="2"/>
-      <c r="H126" s="2"/>
+      <c r="H126" s="2" t="s">
+        <v>145</v>
+      </c>
       <c r="I126" s="2"/>
       <c r="J126" s="2"/>
       <c r="K126" s="3">
@@ -4717,7 +4830,9 @@
         <v>1022</v>
       </c>
       <c r="G127" s="4"/>
-      <c r="H127" s="4"/>
+      <c r="H127" s="4" t="s">
+        <v>145</v>
+      </c>
       <c r="I127" s="4"/>
       <c r="J127" s="4"/>
       <c r="K127" s="5">
@@ -4804,7 +4919,9 @@
         <v>6918</v>
       </c>
       <c r="G138" s="2"/>
-      <c r="H138" s="2"/>
+      <c r="H138" s="2" t="s">
+        <v>152</v>
+      </c>
       <c r="I138" s="2"/>
       <c r="J138" s="2"/>
       <c r="K138" s="3">
@@ -4843,7 +4960,9 @@
         <v>109</v>
       </c>
       <c r="G139" s="4"/>
-      <c r="H139" s="4"/>
+      <c r="H139" s="4" t="s">
+        <v>152</v>
+      </c>
       <c r="I139" s="4"/>
       <c r="J139" s="4"/>
       <c r="K139" s="5">
@@ -4882,7 +5001,9 @@
         <v>7141</v>
       </c>
       <c r="G140" s="2"/>
-      <c r="H140" s="2"/>
+      <c r="H140" s="2" t="s">
+        <v>152</v>
+      </c>
       <c r="I140" s="2"/>
       <c r="J140" s="2"/>
       <c r="K140" s="3">
@@ -4921,7 +5042,9 @@
         <v>136</v>
       </c>
       <c r="G141" s="4"/>
-      <c r="H141" s="4"/>
+      <c r="H141" s="4" t="s">
+        <v>152</v>
+      </c>
       <c r="I141" s="4"/>
       <c r="J141" s="4"/>
       <c r="K141" s="5">
@@ -5020,7 +5143,9 @@
         <v>15828</v>
       </c>
       <c r="G144" s="2"/>
-      <c r="H144" s="2"/>
+      <c r="H144" s="2" t="s">
+        <v>153</v>
+      </c>
       <c r="I144" s="2"/>
       <c r="J144" s="2"/>
       <c r="K144" s="3">
@@ -5059,7 +5184,9 @@
         <v>2006</v>
       </c>
       <c r="G145" s="4"/>
-      <c r="H145" s="4"/>
+      <c r="H145" s="4" t="s">
+        <v>157</v>
+      </c>
       <c r="I145" s="4"/>
       <c r="J145" s="4"/>
       <c r="K145" s="5">
@@ -5098,7 +5225,9 @@
         <v>15464</v>
       </c>
       <c r="G146" s="2"/>
-      <c r="H146" s="2"/>
+      <c r="H146" s="2" t="s">
+        <v>160</v>
+      </c>
       <c r="I146" s="2"/>
       <c r="J146" s="2"/>
       <c r="K146" s="3">
@@ -5137,7 +5266,9 @@
         <v>138</v>
       </c>
       <c r="G147" s="4"/>
-      <c r="H147" s="4"/>
+      <c r="H147" s="4" t="s">
+        <v>159</v>
+      </c>
       <c r="I147" s="4"/>
       <c r="J147" s="4"/>
       <c r="K147" s="5">
@@ -5236,7 +5367,9 @@
         <v>7095</v>
       </c>
       <c r="G150" s="2"/>
-      <c r="H150" s="2"/>
+      <c r="H150" s="2" t="s">
+        <v>154</v>
+      </c>
       <c r="I150" s="2"/>
       <c r="J150" s="2"/>
       <c r="K150" s="3">
@@ -5275,7 +5408,9 @@
         <v>45</v>
       </c>
       <c r="G151" s="4"/>
-      <c r="H151" s="4"/>
+      <c r="H151" s="4" t="s">
+        <v>158</v>
+      </c>
       <c r="I151" s="4"/>
       <c r="J151" s="4"/>
       <c r="K151" s="5">
@@ -5314,7 +5449,9 @@
         <v>7157</v>
       </c>
       <c r="G152" s="2"/>
-      <c r="H152" s="2"/>
+      <c r="H152" s="2" t="s">
+        <v>158</v>
+      </c>
       <c r="I152" s="2"/>
       <c r="J152" s="2"/>
       <c r="K152" s="3">
@@ -5356,7 +5493,7 @@
         <v>96</v>
       </c>
       <c r="H153" s="4" t="s">
-        <v>89</v>
+        <v>158</v>
       </c>
       <c r="I153" s="4"/>
       <c r="J153" s="4"/>
@@ -5456,7 +5593,9 @@
         <v>6953</v>
       </c>
       <c r="G156" s="2"/>
-      <c r="H156" s="2"/>
+      <c r="H156" s="2" t="s">
+        <v>155</v>
+      </c>
       <c r="I156" s="2"/>
       <c r="J156" s="2"/>
       <c r="K156" s="3">
@@ -5495,7 +5634,9 @@
         <v>61</v>
       </c>
       <c r="G157" s="4"/>
-      <c r="H157" s="4"/>
+      <c r="H157" s="4" t="s">
+        <v>155</v>
+      </c>
       <c r="I157" s="4"/>
       <c r="J157" s="4"/>
       <c r="K157" s="5">
@@ -5534,7 +5675,9 @@
         <v>7878</v>
       </c>
       <c r="G158" s="2"/>
-      <c r="H158" s="2"/>
+      <c r="H158" s="2" t="s">
+        <v>156</v>
+      </c>
       <c r="I158" s="2"/>
       <c r="J158" s="2"/>
       <c r="K158" s="3">
@@ -5573,7 +5716,9 @@
         <v>1026</v>
       </c>
       <c r="G159" s="4"/>
-      <c r="H159" s="4"/>
+      <c r="H159" s="4" t="s">
+        <v>155</v>
+      </c>
       <c r="I159" s="4"/>
       <c r="J159" s="4"/>
       <c r="K159" s="5">
@@ -5600,7 +5745,7 @@
       <c r="E160" s="1"/>
       <c r="F160" s="1"/>
       <c r="G160" s="1"/>
-      <c r="H160" s="1"/>
+      <c r="H160" s="8"/>
       <c r="I160" s="1"/>
       <c r="J160" s="1"/>
       <c r="K160" s="1"/>
@@ -5672,7 +5817,9 @@
         <v>7207</v>
       </c>
       <c r="G162" s="2"/>
-      <c r="H162" s="2"/>
+      <c r="H162" s="2" t="s">
+        <v>156</v>
+      </c>
       <c r="I162" s="2"/>
       <c r="J162" s="2"/>
       <c r="K162" s="3">
@@ -5711,7 +5858,9 @@
         <v>1278</v>
       </c>
       <c r="G163" s="4"/>
-      <c r="H163" s="4"/>
+      <c r="H163" s="4" t="s">
+        <v>156</v>
+      </c>
       <c r="I163" s="4"/>
       <c r="J163" s="4"/>
       <c r="K163" s="5">
@@ -5750,7 +5899,9 @@
         <v>7207</v>
       </c>
       <c r="G164" s="2"/>
-      <c r="H164" s="2"/>
+      <c r="H164" s="2" t="s">
+        <v>156</v>
+      </c>
       <c r="I164" s="2"/>
       <c r="J164" s="2"/>
       <c r="K164" s="3">
@@ -5789,7 +5940,9 @@
         <v>1273</v>
       </c>
       <c r="G165" s="4"/>
-      <c r="H165" s="4"/>
+      <c r="H165" s="4" t="s">
+        <v>156</v>
+      </c>
       <c r="I165" s="4"/>
       <c r="J165" s="4"/>
       <c r="K165" s="5">

</xml_diff>

<commit_message>
added LLM as a judge
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/21c1a4ced64a9754/Documents/Uni/Bachelor Thesis/BachelorThesis/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vanessa\Documents\Uni\Bachelor-Thesis\BachelorThesis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="341" documentId="13_ncr:1_{30350997-3BBF-49AB-916C-212AA2CBCFFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{86315208-3E9E-4B82-8859-205CA8B4FD4B}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC4504C3-57EE-4E26-A35F-7C2746216775}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12390" yWindow="0" windowWidth="12660" windowHeight="16010" xr2:uid="{2A4234DB-3A22-4351-83C3-53CA1AE1142A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{2A4234DB-3A22-4351-83C3-53CA1AE1142A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="773" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="163">
   <si>
     <t>Benchmarking results LLMs</t>
   </si>
@@ -519,6 +519,12 @@
   </si>
   <si>
     <t>precomputation with brute force filtering</t>
+  </si>
+  <si>
+    <t>PART B</t>
+  </si>
+  <si>
+    <t>PART A</t>
   </si>
 </sst>
 </file>
@@ -632,10 +638,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -956,19 +958,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9626A942-19B5-4B39-BBE2-849051787A6F}">
   <dimension ref="A1:O184"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="5" max="5" width="15.26953125" customWidth="1"/>
-    <col min="6" max="6" width="15.1796875" customWidth="1"/>
-    <col min="8" max="8" width="50.1796875" customWidth="1"/>
-    <col min="11" max="11" width="13.81640625" customWidth="1"/>
-    <col min="12" max="12" width="12.81640625" customWidth="1"/>
-    <col min="14" max="14" width="14.453125" customWidth="1"/>
-    <col min="15" max="15" width="14.81640625" customWidth="1"/>
-    <col min="16" max="16" width="13.7265625" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" customWidth="1"/>
+    <col min="6" max="6" width="15.140625" customWidth="1"/>
+    <col min="8" max="8" width="50.140625" customWidth="1"/>
+    <col min="11" max="11" width="13.85546875" customWidth="1"/>
+    <col min="12" max="12" width="12.85546875" customWidth="1"/>
+    <col min="14" max="14" width="14.42578125" customWidth="1"/>
+    <col min="15" max="15" width="14.85546875" customWidth="1"/>
+    <col min="16" max="16" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -979,12 +981,17 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2024</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
@@ -1027,7 +1034,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
@@ -1070,7 +1077,7 @@
         <v>7004</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>9</v>
       </c>
@@ -1113,7 +1120,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>9</v>
       </c>
@@ -1156,7 +1163,7 @@
         <v>7328</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>9</v>
       </c>
@@ -1199,7 +1206,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -1216,7 +1223,7 @@
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>1</v>
       </c>
@@ -1259,7 +1266,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>23</v>
       </c>
@@ -1302,7 +1309,7 @@
         <v>6961</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
         <v>23</v>
       </c>
@@ -1345,7 +1352,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -1388,7 +1395,7 @@
         <v>7055</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>23</v>
       </c>
@@ -1431,7 +1438,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -1448,7 +1455,7 @@
       <c r="N17" s="1"/>
       <c r="O17" s="1"/>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>1</v>
       </c>
@@ -1491,7 +1498,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>24</v>
       </c>
@@ -1534,7 +1541,7 @@
         <v>7141</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>24</v>
       </c>
@@ -1577,7 +1584,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>24</v>
       </c>
@@ -1620,7 +1627,7 @@
         <v>7117</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
         <v>24</v>
       </c>
@@ -1663,7 +1670,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -1680,7 +1687,7 @@
       <c r="N23" s="1"/>
       <c r="O23" s="1"/>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>1</v>
       </c>
@@ -1723,7 +1730,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>25</v>
       </c>
@@ -1766,7 +1773,7 @@
         <v>7172</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
         <v>25</v>
       </c>
@@ -1809,7 +1816,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>25</v>
       </c>
@@ -1852,7 +1859,7 @@
         <v>7602</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
         <v>25</v>
       </c>
@@ -1895,7 +1902,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -1912,7 +1919,7 @@
       <c r="N29" s="1"/>
       <c r="O29" s="1"/>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>1</v>
       </c>
@@ -1955,7 +1962,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>26</v>
       </c>
@@ -1998,7 +2005,7 @@
         <v>7078</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
         <v>26</v>
       </c>
@@ -2041,7 +2048,7 @@
         <v>1031</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>26</v>
       </c>
@@ -2084,7 +2091,7 @@
         <v>7121</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
         <v>26</v>
       </c>
@@ -2127,7 +2134,7 @@
         <v>1039</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
@@ -2144,7 +2151,7 @@
       <c r="N35" s="1"/>
       <c r="O35" s="1"/>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>1</v>
       </c>
@@ -2187,7 +2194,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>27</v>
       </c>
@@ -2230,7 +2237,7 @@
         <v>7078</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
         <v>27</v>
       </c>
@@ -2273,7 +2280,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>27</v>
       </c>
@@ -2316,7 +2323,7 @@
         <v>7074</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
         <v>27</v>
       </c>
@@ -2359,12 +2366,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>2025</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>1</v>
       </c>
@@ -2407,7 +2414,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>9</v>
       </c>
@@ -2450,7 +2457,7 @@
         <v>6934</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
         <v>9</v>
       </c>
@@ -2493,7 +2500,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>9</v>
       </c>
@@ -2536,7 +2543,7 @@
         <v>7180</v>
       </c>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
         <v>9</v>
       </c>
@@ -2579,7 +2586,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="1"/>
       <c r="B55" s="1"/>
       <c r="C55" s="1"/>
@@ -2596,7 +2603,7 @@
       <c r="N55" s="1"/>
       <c r="O55" s="1"/>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>1</v>
       </c>
@@ -2639,7 +2646,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>23</v>
       </c>
@@ -2682,7 +2689,7 @@
         <v>7012</v>
       </c>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
         <v>23</v>
       </c>
@@ -2725,7 +2732,7 @@
         <v>2004</v>
       </c>
     </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>23</v>
       </c>
@@ -2768,7 +2775,7 @@
         <v>10863</v>
       </c>
     </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
         <v>23</v>
       </c>
@@ -2811,7 +2818,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="1"/>
       <c r="B61" s="1"/>
       <c r="C61" s="1"/>
@@ -2828,7 +2835,7 @@
       <c r="N61" s="1"/>
       <c r="O61" s="1"/>
     </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>1</v>
       </c>
@@ -2871,7 +2878,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>53</v>
       </c>
@@ -2914,7 +2921,7 @@
         <v>7102</v>
       </c>
     </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
         <v>53</v>
       </c>
@@ -2957,7 +2964,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>53</v>
       </c>
@@ -3000,7 +3007,7 @@
         <v>7191</v>
       </c>
     </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
         <v>53</v>
       </c>
@@ -3043,7 +3050,7 @@
         <v>1027</v>
       </c>
     </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="1"/>
       <c r="B67" s="1"/>
       <c r="C67" s="1"/>
@@ -3060,7 +3067,7 @@
       <c r="N67" s="1"/>
       <c r="O67" s="1"/>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>1</v>
       </c>
@@ -3103,7 +3110,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
         <v>54</v>
       </c>
@@ -3146,7 +3153,7 @@
         <v>6980</v>
       </c>
     </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
         <v>54</v>
       </c>
@@ -3189,7 +3196,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>54</v>
       </c>
@@ -3232,7 +3239,7 @@
         <v>7938</v>
       </c>
     </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
         <v>54</v>
       </c>
@@ -3275,7 +3282,7 @@
         <v>1047</v>
       </c>
     </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A73" s="1"/>
       <c r="B73" s="1"/>
       <c r="C73" s="1"/>
@@ -3292,7 +3299,7 @@
       <c r="N73" s="1"/>
       <c r="O73" s="1"/>
     </row>
-    <row r="74" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>1</v>
       </c>
@@ -3335,7 +3342,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
         <v>55</v>
       </c>
@@ -3378,7 +3385,7 @@
         <v>7105</v>
       </c>
     </row>
-    <row r="76" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
         <v>55</v>
       </c>
@@ -3421,7 +3428,7 @@
         <v>1152</v>
       </c>
     </row>
-    <row r="77" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>55</v>
       </c>
@@ -3464,7 +3471,7 @@
         <v>7098</v>
       </c>
     </row>
-    <row r="78" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
         <v>55</v>
       </c>
@@ -3507,7 +3514,7 @@
         <v>1148</v>
       </c>
     </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
       <c r="C79" s="1"/>
@@ -3524,7 +3531,7 @@
       <c r="N79" s="1"/>
       <c r="O79" s="1"/>
     </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>1</v>
       </c>
@@ -3567,7 +3574,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="81" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
         <v>24</v>
       </c>
@@ -3610,7 +3617,7 @@
         <v>7156</v>
       </c>
     </row>
-    <row r="82" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
         <v>24</v>
       </c>
@@ -3653,7 +3660,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="83" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
         <v>24</v>
       </c>
@@ -3696,7 +3703,7 @@
         <v>7160</v>
       </c>
     </row>
-    <row r="84" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A84" s="4" t="s">
         <v>24</v>
       </c>
@@ -3739,17 +3746,22 @@
         <v>78</v>
       </c>
     </row>
-    <row r="96" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B92" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="96" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="97" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>2024</v>
       </c>
     </row>
-    <row r="99" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>1</v>
       </c>
@@ -3792,7 +3804,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="100" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
         <v>9</v>
       </c>
@@ -3833,7 +3845,7 @@
         <v>6980</v>
       </c>
     </row>
-    <row r="101" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A101" s="4" t="s">
         <v>9</v>
       </c>
@@ -3874,7 +3886,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="102" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
         <v>9</v>
       </c>
@@ -3915,7 +3927,7 @@
         <v>7301</v>
       </c>
     </row>
-    <row r="103" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A103" s="4" t="s">
         <v>9</v>
       </c>
@@ -3956,7 +3968,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="104" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A104" s="1"/>
       <c r="B104" s="1"/>
       <c r="C104" s="1"/>
@@ -3973,7 +3985,7 @@
       <c r="N104" s="1"/>
       <c r="O104" s="1"/>
     </row>
-    <row r="105" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
         <v>1</v>
       </c>
@@ -4016,7 +4028,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="106" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
         <v>23</v>
       </c>
@@ -4057,7 +4069,7 @@
         <v>6969</v>
       </c>
     </row>
-    <row r="107" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A107" s="4" t="s">
         <v>23</v>
       </c>
@@ -4098,7 +4110,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="108" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
         <v>23</v>
       </c>
@@ -4139,7 +4151,7 @@
         <v>7031</v>
       </c>
     </row>
-    <row r="109" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A109" s="4" t="s">
         <v>23</v>
       </c>
@@ -4179,7 +4191,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="110" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A110" s="1"/>
       <c r="B110" s="1"/>
       <c r="C110" s="1"/>
@@ -4196,7 +4208,7 @@
       <c r="N110" s="1"/>
       <c r="O110" s="1"/>
     </row>
-    <row r="111" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
         <v>1</v>
       </c>
@@ -4239,7 +4251,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="112" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
         <v>24</v>
       </c>
@@ -4280,7 +4292,7 @@
         <v>7203</v>
       </c>
     </row>
-    <row r="113" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A113" s="4" t="s">
         <v>24</v>
       </c>
@@ -4321,7 +4333,7 @@
         <v>1004</v>
       </c>
     </row>
-    <row r="114" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
         <v>24</v>
       </c>
@@ -4362,7 +4374,7 @@
         <v>7125</v>
       </c>
     </row>
-    <row r="115" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A115" s="4" t="s">
         <v>24</v>
       </c>
@@ -4403,7 +4415,7 @@
         <v>1004</v>
       </c>
     </row>
-    <row r="116" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A116" s="1"/>
       <c r="B116" s="1"/>
       <c r="C116" s="1"/>
@@ -4420,7 +4432,7 @@
       <c r="N116" s="1"/>
       <c r="O116" s="1"/>
     </row>
-    <row r="117" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
         <v>1</v>
       </c>
@@ -4463,7 +4475,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="118" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
         <v>25</v>
       </c>
@@ -4504,7 +4516,7 @@
         <v>7375</v>
       </c>
     </row>
-    <row r="119" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A119" s="4" t="s">
         <v>25</v>
       </c>
@@ -4545,7 +4557,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="120" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
         <v>25</v>
       </c>
@@ -4586,7 +4598,7 @@
         <v>7520</v>
       </c>
     </row>
-    <row r="121" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A121" s="4" t="s">
         <v>25</v>
       </c>
@@ -4627,7 +4639,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="122" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A122" s="1"/>
       <c r="B122" s="1"/>
       <c r="C122" s="1"/>
@@ -4644,7 +4656,7 @@
       <c r="N122" s="1"/>
       <c r="O122" s="1"/>
     </row>
-    <row r="123" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A123" s="1" t="s">
         <v>1</v>
       </c>
@@ -4687,7 +4699,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="124" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
         <v>26</v>
       </c>
@@ -4728,7 +4740,7 @@
         <v>7203</v>
       </c>
     </row>
-    <row r="125" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A125" s="4" t="s">
         <v>26</v>
       </c>
@@ -4769,7 +4781,7 @@
         <v>1094</v>
       </c>
     </row>
-    <row r="126" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
         <v>26</v>
       </c>
@@ -4810,7 +4822,7 @@
         <v>7594</v>
       </c>
     </row>
-    <row r="127" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A127" s="4" t="s">
         <v>26</v>
       </c>
@@ -4851,12 +4863,12 @@
         <v>1020</v>
       </c>
     </row>
-    <row r="135" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>2025</v>
       </c>
     </row>
-    <row r="137" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A137" s="1" t="s">
         <v>1</v>
       </c>
@@ -4899,7 +4911,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="138" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
         <v>9</v>
       </c>
@@ -4940,7 +4952,7 @@
         <v>6914</v>
       </c>
     </row>
-    <row r="139" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A139" s="4" t="s">
         <v>9</v>
       </c>
@@ -4981,7 +4993,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="140" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
         <v>9</v>
       </c>
@@ -5022,7 +5034,7 @@
         <v>7137</v>
       </c>
     </row>
-    <row r="141" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A141" s="4" t="s">
         <v>9</v>
       </c>
@@ -5063,7 +5075,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="142" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A142" s="1"/>
       <c r="B142" s="1"/>
       <c r="C142" s="1"/>
@@ -5080,7 +5092,7 @@
       <c r="N142" s="1"/>
       <c r="O142" s="1"/>
     </row>
-    <row r="143" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A143" s="1" t="s">
         <v>1</v>
       </c>
@@ -5123,7 +5135,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="144" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
         <v>23</v>
       </c>
@@ -5164,7 +5176,7 @@
         <v>15824</v>
       </c>
     </row>
-    <row r="145" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A145" s="4" t="s">
         <v>23</v>
       </c>
@@ -5205,7 +5217,7 @@
         <v>2004</v>
       </c>
     </row>
-    <row r="146" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
         <v>23</v>
       </c>
@@ -5246,7 +5258,7 @@
         <v>15457</v>
       </c>
     </row>
-    <row r="147" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A147" s="4" t="s">
         <v>23</v>
       </c>
@@ -5287,7 +5299,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="148" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A148" s="1"/>
       <c r="B148" s="1"/>
       <c r="C148" s="1"/>
@@ -5304,7 +5316,7 @@
       <c r="N148" s="1"/>
       <c r="O148" s="1"/>
     </row>
-    <row r="149" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A149" s="1" t="s">
         <v>1</v>
       </c>
@@ -5347,7 +5359,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="150" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
         <v>53</v>
       </c>
@@ -5388,7 +5400,7 @@
         <v>7094</v>
       </c>
     </row>
-    <row r="151" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A151" s="4" t="s">
         <v>53</v>
       </c>
@@ -5429,7 +5441,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="152" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
         <v>53</v>
       </c>
@@ -5470,7 +5482,7 @@
         <v>7156</v>
       </c>
     </row>
-    <row r="153" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A153" s="4" t="s">
         <v>53</v>
       </c>
@@ -5513,7 +5525,7 @@
         <v>1016</v>
       </c>
     </row>
-    <row r="154" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A154" s="1"/>
       <c r="B154" s="1"/>
       <c r="C154" s="1"/>
@@ -5530,7 +5542,7 @@
       <c r="N154" s="1"/>
       <c r="O154" s="1"/>
     </row>
-    <row r="155" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A155" s="1" t="s">
         <v>1</v>
       </c>
@@ -5573,7 +5585,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="156" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
         <v>54</v>
       </c>
@@ -5614,7 +5626,7 @@
         <v>6949</v>
       </c>
     </row>
-    <row r="157" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A157" s="4" t="s">
         <v>54</v>
       </c>
@@ -5655,7 +5667,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="158" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
         <v>54</v>
       </c>
@@ -5696,7 +5708,7 @@
         <v>7875</v>
       </c>
     </row>
-    <row r="159" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A159" s="4" t="s">
         <v>54</v>
       </c>
@@ -5737,7 +5749,7 @@
         <v>1023</v>
       </c>
     </row>
-    <row r="160" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A160" s="1"/>
       <c r="B160" s="1"/>
       <c r="C160" s="1"/>
@@ -5754,7 +5766,7 @@
       <c r="N160" s="1"/>
       <c r="O160" s="1"/>
     </row>
-    <row r="161" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A161" s="1" t="s">
         <v>1</v>
       </c>
@@ -5797,7 +5809,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="162" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
         <v>55</v>
       </c>
@@ -5838,7 +5850,7 @@
         <v>7203</v>
       </c>
     </row>
-    <row r="163" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A163" s="4" t="s">
         <v>55</v>
       </c>
@@ -5879,7 +5891,7 @@
         <v>1273</v>
       </c>
     </row>
-    <row r="164" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A164" s="2" t="s">
         <v>55</v>
       </c>
@@ -5920,7 +5932,7 @@
         <v>7203</v>
       </c>
     </row>
-    <row r="165" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A165" s="4" t="s">
         <v>55</v>
       </c>
@@ -5961,7 +5973,7 @@
         <v>1270</v>
       </c>
     </row>
-    <row r="166" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A166" s="1"/>
       <c r="B166" s="1"/>
       <c r="C166" s="1"/>
@@ -5978,12 +5990,12 @@
       <c r="N166" s="1"/>
       <c r="O166" s="1"/>
     </row>
-    <row r="183" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="184" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A184">
         <v>2024</v>
       </c>

</xml_diff>